<commit_message>
M6 step 2: ABC classes with nested IF and COUNTIF summary (A 60, B 34, C 26; check total 120)
</commit_message>
<xml_diff>
--- a/excel/Spend_Analysis.xlsx
+++ b/excel/Spend_Analysis.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2CE5B02-FECB-D343-8209-875965449C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B97F94-08BF-8B4F-BA3C-1F4F66E5B685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suppliers" sheetId="1" r:id="rId1"/>
-    <sheet name="Terms" sheetId="2" r:id="rId2"/>
-    <sheet name="Settings" sheetId="3" r:id="rId3"/>
+    <sheet name="Results" sheetId="4" r:id="rId2"/>
+    <sheet name="Terms" sheetId="2" r:id="rId3"/>
+    <sheet name="Settings" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="303">
   <si>
     <t>Golden ID</t>
   </si>
@@ -923,6 +924,27 @@
   </si>
   <si>
     <t>Cumulative share</t>
+  </si>
+  <si>
+    <t>ABC class</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Suppliers</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -1004,7 +1026,10 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="13" formatCode="0%"/>
     </dxf>
@@ -1022,12 +1047,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSpend" displayName="tblSpend" ref="A1:K121">
-  <autoFilter ref="A1:K121" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSpend" displayName="tblSpend" ref="A1:L121">
+  <autoFilter ref="A1:L121" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I121">
     <sortCondition descending="1" ref="F1:F121"/>
   </sortState>
-  <tableColumns count="11">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Golden ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Supplier"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Country"/>
@@ -1040,8 +1065,11 @@
     <tableColumn id="10" xr3:uid="{5D1E5103-053F-9149-A678-5C4D8626A5EA}" name="Spend share" dataCellStyle="Percent">
       <calculatedColumnFormula>F2/SUM($F$2:$F$121)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{B3C0593A-4800-A24E-858E-2C3789403277}" name="Cumulative share" dataDxfId="0">
+    <tableColumn id="11" xr3:uid="{B3C0593A-4800-A24E-858E-2C3789403277}" name="Cumulative share" dataDxfId="1">
       <calculatedColumnFormula>SUM($J$2:J2)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{DFA46FC0-C59B-9B4C-8696-052595BBF44D}" name="ABC class" dataDxfId="0">
+      <calculatedColumnFormula>IF(K2&lt;=80%,"A",IF(K2&lt;=95%,"B","C"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1333,7 +1361,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
@@ -1346,9 +1374,10 @@
     <col min="9" max="9" width="16.1640625" customWidth="1"/>
     <col min="10" max="10" width="15" style="7" customWidth="1"/>
     <col min="11" max="11" width="18.6640625" customWidth="1"/>
+    <col min="12" max="12" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1382,8 +1411,11 @@
       <c r="K1" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>228</v>
       </c>
@@ -1419,8 +1451,12 @@
         <f>SUM($J$2:J2)</f>
         <v>2.9880261291344874E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" t="str">
+        <f t="shared" ref="L2:L33" si="1">IF(K2&lt;=80%,"A",IF(K2&lt;=95%,"B","C"))</f>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>61</v>
       </c>
@@ -1456,8 +1492,12 @@
         <f>SUM($J$2:J3)</f>
         <v>5.7832973581577421E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>236</v>
       </c>
@@ -1493,8 +1533,12 @@
         <f>SUM($J$2:J4)</f>
         <v>8.4849243388326029E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>136</v>
       </c>
@@ -1530,8 +1574,12 @@
         <f>SUM($J$2:J5)</f>
         <v>0.10982803026881408</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L5" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -1567,8 +1615,12 @@
         <f>SUM($J$2:J6)</f>
         <v>0.13384496632984735</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L6" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>198</v>
       </c>
@@ -1604,8 +1656,12 @@
         <f>SUM($J$2:J7)</f>
         <v>0.15640556968660585</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L7" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>238</v>
       </c>
@@ -1641,8 +1697,12 @@
         <f>SUM($J$2:J8)</f>
         <v>0.17868487746878758</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L8" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>120</v>
       </c>
@@ -1678,8 +1738,12 @@
         <f>SUM($J$2:J9)</f>
         <v>0.20090641320536567</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>158</v>
       </c>
@@ -1715,8 +1779,12 @@
         <f>SUM($J$2:J10)</f>
         <v>0.22289901719919805</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>220</v>
       </c>
@@ -1752,8 +1820,12 @@
         <f>SUM($J$2:J11)</f>
         <v>0.24368475432923664</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -1789,8 +1861,12 @@
         <f>SUM($J$2:J12)</f>
         <v>0.26411712972471868</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>266</v>
       </c>
@@ -1826,8 +1902,12 @@
         <f>SUM($J$2:J13)</f>
         <v>0.28436482488862719</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>206</v>
       </c>
@@ -1863,8 +1943,12 @@
         <f>SUM($J$2:J14)</f>
         <v>0.3042301969909349</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>180</v>
       </c>
@@ -1900,8 +1984,12 @@
         <f>SUM($J$2:J15)</f>
         <v>0.32315503964314829</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>260</v>
       </c>
@@ -1937,8 +2025,12 @@
         <f>SUM($J$2:J16)</f>
         <v>0.33989779468616643</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>172</v>
       </c>
@@ -1974,8 +2066,12 @@
         <f>SUM($J$2:J17)</f>
         <v>0.35662327082847317</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>76</v>
       </c>
@@ -2011,8 +2107,12 @@
         <f>SUM($J$2:J18)</f>
         <v>0.37248901554986397</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -2048,8 +2148,12 @@
         <f>SUM($J$2:J19)</f>
         <v>0.3879850712077772</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>128</v>
       </c>
@@ -2085,8 +2189,12 @@
         <f>SUM($J$2:J20)</f>
         <v>0.40344441262459879</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>148</v>
       </c>
@@ -2122,8 +2230,12 @@
         <f>SUM($J$2:J21)</f>
         <v>0.41752119895717998</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L21" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>192</v>
       </c>
@@ -2159,8 +2271,12 @@
         <f>SUM($J$2:J22)</f>
         <v>0.43124647877790384</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>196</v>
       </c>
@@ -2196,8 +2312,12 @@
         <f>SUM($J$2:J23)</f>
         <v>0.4445999883997237</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>15</v>
       </c>
@@ -2233,8 +2353,12 @@
         <f>SUM($J$2:J24)</f>
         <v>0.4577812977566883</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>234</v>
       </c>
@@ -2270,8 +2394,12 @@
         <f>SUM($J$2:J25)</f>
         <v>0.47075529111139697</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>268</v>
       </c>
@@ -2307,8 +2435,12 @@
         <f>SUM($J$2:J26)</f>
         <v>0.48331577517938967</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>190</v>
       </c>
@@ -2344,8 +2476,12 @@
         <f>SUM($J$2:J27)</f>
         <v>0.49550124412021479</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L27" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>80</v>
       </c>
@@ -2381,8 +2517,12 @@
         <f>SUM($J$2:J28)</f>
         <v>0.50744661917581801</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L28" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>96</v>
       </c>
@@ -2418,8 +2558,12 @@
         <f>SUM($J$2:J29)</f>
         <v>0.51929262686065014</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L29" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>202</v>
       </c>
@@ -2455,8 +2599,12 @@
         <f>SUM($J$2:J30)</f>
         <v>0.53103308538099403</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L30" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -2492,8 +2640,12 @@
         <f>SUM($J$2:J31)</f>
         <v>0.54231375673474502</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L31" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>106</v>
       </c>
@@ -2529,8 +2681,12 @@
         <f>SUM($J$2:J32)</f>
         <v>0.55294093102708153</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L32" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>204</v>
       </c>
@@ -2566,8 +2722,12 @@
         <f>SUM($J$2:J33)</f>
         <v>0.56351988322091917</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L33" t="str">
+        <f t="shared" si="1"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>88</v>
       </c>
@@ -2596,15 +2756,19 @@
         <v>25</v>
       </c>
       <c r="J34" s="7">
-        <f t="shared" ref="J34:J65" si="1">F34/SUM($F$2:$F$121)</f>
+        <f t="shared" ref="J34:J65" si="2">F34/SUM($F$2:$F$121)</f>
         <v>1.0373135430589573E-2</v>
       </c>
       <c r="K34" s="4">
         <f>SUM($J$2:J34)</f>
         <v>0.57389301865150877</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L34" t="str">
+        <f t="shared" ref="L34:L65" si="3">IF(K34&lt;=80%,"A",IF(K34&lt;=95%,"B","C"))</f>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>59</v>
       </c>
@@ -2633,15 +2797,19 @@
         <v>25</v>
       </c>
       <c r="J35" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.0129108610162139E-2</v>
       </c>
       <c r="K35" s="4">
         <f>SUM($J$2:J35)</f>
         <v>0.58402212726167091</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L35" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -2670,15 +2838,19 @@
         <v>20</v>
       </c>
       <c r="J36" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.0073763414915953E-2</v>
       </c>
       <c r="K36" s="4">
         <f>SUM($J$2:J36)</f>
         <v>0.59409589067658686</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L36" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>214</v>
       </c>
@@ -2707,15 +2879,19 @@
         <v>25</v>
       </c>
       <c r="J37" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.000662283697335E-2</v>
       </c>
       <c r="K37" s="4">
         <f>SUM($J$2:J37)</f>
         <v>0.60410251351356026</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L37" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>26</v>
       </c>
@@ -2744,15 +2920,19 @@
         <v>30</v>
       </c>
       <c r="J38" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.8667452067095467E-3</v>
       </c>
       <c r="K38" s="4">
         <f>SUM($J$2:J38)</f>
         <v>0.61396925872026975</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L38" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -2781,15 +2961,19 @@
         <v>30</v>
       </c>
       <c r="J39" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.8295038359210926E-3</v>
       </c>
       <c r="K39" s="4">
         <f>SUM($J$2:J39)</f>
         <v>0.62379876255619082</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L39" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>150</v>
       </c>
@@ -2818,15 +3002,19 @@
         <v>25</v>
       </c>
       <c r="J40" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.8080352809959831E-3</v>
       </c>
       <c r="K40" s="4">
         <f>SUM($J$2:J40)</f>
         <v>0.63360679783718676</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L40" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -2855,15 +3043,19 @@
         <v>20</v>
       </c>
       <c r="J41" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.6698793795471239E-3</v>
       </c>
       <c r="K41" s="4">
         <f>SUM($J$2:J41)</f>
         <v>0.64327667721673387</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L41" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>132</v>
       </c>
@@ -2892,15 +3084,19 @@
         <v>30</v>
       </c>
       <c r="J42" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9.2346995856195796E-3</v>
       </c>
       <c r="K42" s="4">
         <f>SUM($J$2:J42)</f>
         <v>0.65251137680235349</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L42" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>154</v>
       </c>
@@ -2929,15 +3125,19 @@
         <v>20</v>
       </c>
       <c r="J43" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.9998667286055462E-3</v>
       </c>
       <c r="K43" s="4">
         <f>SUM($J$2:J43)</f>
         <v>0.66151124353095903</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L43" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>92</v>
       </c>
@@ -2966,15 +3166,19 @@
         <v>20</v>
       </c>
       <c r="J44" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.4996240692417034E-3</v>
       </c>
       <c r="K44" s="4">
         <f>SUM($J$2:J44)</f>
         <v>0.67001086760020068</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L44" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -3003,15 +3207,19 @@
         <v>45</v>
       </c>
       <c r="J45" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.4436456337753079E-3</v>
       </c>
       <c r="K45" s="4">
         <f>SUM($J$2:J45)</f>
         <v>0.67845451323397599</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L45" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>102</v>
       </c>
@@ -3040,15 +3248,19 @@
         <v>30</v>
       </c>
       <c r="J46" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.3354471291224551E-3</v>
       </c>
       <c r="K46" s="4">
         <f>SUM($J$2:J46)</f>
         <v>0.68678996036309847</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L46" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>258</v>
       </c>
@@ -3077,15 +3289,19 @@
         <v>45</v>
       </c>
       <c r="J47" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.9611953131392566E-3</v>
       </c>
       <c r="K47" s="4">
         <f>SUM($J$2:J47)</f>
         <v>0.69475115567623769</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L47" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>110</v>
       </c>
@@ -3114,15 +3330,19 @@
         <v>20</v>
       </c>
       <c r="J48" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.9223725532603373E-3</v>
       </c>
       <c r="K48" s="4">
         <f>SUM($J$2:J48)</f>
         <v>0.70267352822949802</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L48" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>134</v>
       </c>
@@ -3151,15 +3371,19 @@
         <v>14</v>
       </c>
       <c r="J49" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.8885677942615532E-3</v>
       </c>
       <c r="K49" s="4">
         <f>SUM($J$2:J49)</f>
         <v>0.71056209602375953</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L49" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>94</v>
       </c>
@@ -3188,15 +3412,19 @@
         <v>20</v>
       </c>
       <c r="J50" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.7195953430692701E-3</v>
       </c>
       <c r="K50" s="4">
         <f>SUM($J$2:J50)</f>
         <v>0.71828169136682884</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L50" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>73</v>
       </c>
@@ -3225,15 +3453,19 @@
         <v>45</v>
       </c>
       <c r="J51" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.6512841264493089E-3</v>
       </c>
       <c r="K51" s="4">
         <f>SUM($J$2:J51)</f>
         <v>0.72593297549327818</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L51" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>114</v>
       </c>
@@ -3262,15 +3494,19 @@
         <v>30</v>
       </c>
       <c r="J52" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.2846619993895906E-3</v>
       </c>
       <c r="K52" s="4">
         <f>SUM($J$2:J52)</f>
         <v>0.73321763749266777</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L52" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>86</v>
       </c>
@@ -3299,15 +3535,19 @@
         <v>20</v>
       </c>
       <c r="J53" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.2541535124559979E-3</v>
       </c>
       <c r="K53" s="4">
         <f>SUM($J$2:J53)</f>
         <v>0.74047179100512373</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L53" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>250</v>
       </c>
@@ -3336,15 +3576,19 @@
         <v>20</v>
       </c>
       <c r="J54" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.1764121509350996E-3</v>
       </c>
       <c r="K54" s="4">
         <f>SUM($J$2:J54)</f>
         <v>0.74764820315605884</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L54" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>226</v>
       </c>
@@ -3373,15 +3617,19 @@
         <v>30</v>
       </c>
       <c r="J55" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.1143066884731777E-3</v>
       </c>
       <c r="K55" s="4">
         <f>SUM($J$2:J55)</f>
         <v>0.75476250984453197</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L55" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>272</v>
       </c>
@@ -3410,15 +3658,19 @@
         <v>25</v>
       </c>
       <c r="J56" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.0400806659044624E-3</v>
       </c>
       <c r="K56" s="4">
         <f>SUM($J$2:J56)</f>
         <v>0.76180259051043642</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L56" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>176</v>
       </c>
@@ -3447,15 +3699,19 @@
         <v>45</v>
       </c>
       <c r="J57" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.0288432191858508E-3</v>
       </c>
       <c r="K57" s="4">
         <f>SUM($J$2:J57)</f>
         <v>0.76883143372962226</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L57" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>252</v>
       </c>
@@ -3484,15 +3740,19 @@
         <v>45</v>
       </c>
       <c r="J58" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.796057268397139E-3</v>
       </c>
       <c r="K58" s="4">
         <f>SUM($J$2:J58)</f>
         <v>0.77562749099801942</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L58" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>90</v>
       </c>
@@ -3521,15 +3781,19 @@
         <v>20</v>
       </c>
       <c r="J59" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.745267979816341E-3</v>
       </c>
       <c r="K59" s="4">
         <f>SUM($J$2:J59)</f>
         <v>0.78237275897783576</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L59" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>54</v>
       </c>
@@ -3558,15 +3822,19 @@
         <v>30</v>
       </c>
       <c r="J60" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.56914847143598E-3</v>
       </c>
       <c r="K60" s="4">
         <f>SUM($J$2:J60)</f>
         <v>0.78894190744927173</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L60" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>164</v>
       </c>
@@ -3595,15 +3863,19 @@
         <v>25</v>
       </c>
       <c r="J61" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.5622170582147832E-3</v>
       </c>
       <c r="K61" s="4">
         <f>SUM($J$2:J61)</f>
         <v>0.79550412450748653</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L61" t="str">
+        <f t="shared" si="3"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>168</v>
       </c>
@@ -3632,15 +3904,19 @@
         <v>20</v>
       </c>
       <c r="J62" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.4312835181964062E-3</v>
       </c>
       <c r="K62" s="4">
         <f>SUM($J$2:J62)</f>
         <v>0.80193540802568297</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L62" t="str">
+        <f t="shared" si="3"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>100</v>
       </c>
@@ -3669,15 +3945,19 @@
         <v>20</v>
       </c>
       <c r="J63" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.4017163342928521E-3</v>
       </c>
       <c r="K63" s="4">
         <f>SUM($J$2:J63)</f>
         <v>0.80833712435997584</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L63" t="str">
+        <f t="shared" si="3"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -3706,15 +3986,19 @@
         <v>25</v>
       </c>
       <c r="J64" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.3790463344094023E-3</v>
       </c>
       <c r="K64" s="4">
         <f>SUM($J$2:J64)</f>
         <v>0.81471617069438529</v>
       </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L64" t="str">
+        <f t="shared" si="3"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>188</v>
       </c>
@@ -3743,15 +4027,19 @@
         <v>30</v>
       </c>
       <c r="J65" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6.2261889910913883E-3</v>
       </c>
       <c r="K65" s="4">
         <f>SUM($J$2:J65)</f>
         <v>0.82094235968547669</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L65" t="str">
+        <f t="shared" si="3"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>216</v>
       </c>
@@ -3780,15 +4068,19 @@
         <v>25</v>
       </c>
       <c r="J66" s="7">
-        <f t="shared" ref="J66:J97" si="2">F66/SUM($F$2:$F$121)</f>
+        <f t="shared" ref="J66:J97" si="4">F66/SUM($F$2:$F$121)</f>
         <v>6.0938486309081163E-3</v>
       </c>
       <c r="K66" s="4">
         <f>SUM($J$2:J66)</f>
         <v>0.8270362083163848</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L66" t="str">
+        <f t="shared" ref="L66:L97" si="5">IF(K66&lt;=80%,"A",IF(K66&lt;=95%,"B","C"))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>246</v>
       </c>
@@ -3817,15 +4109,19 @@
         <v>25</v>
       </c>
       <c r="J67" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.9128206550911151E-3</v>
       </c>
       <c r="K67" s="4">
         <f>SUM($J$2:J67)</f>
         <v>0.83294902897147594</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L67" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>152</v>
       </c>
@@ -3854,15 +4150,19 @@
         <v>20</v>
       </c>
       <c r="J68" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.8867859247402898E-3</v>
       </c>
       <c r="K68" s="4">
         <f>SUM($J$2:J68)</f>
         <v>0.83883581489621628</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L68" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>210</v>
       </c>
@@ -3891,15 +4191,19 @@
         <v>25</v>
       </c>
       <c r="J69" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.7980501438285358E-3</v>
       </c>
       <c r="K69" s="4">
         <f>SUM($J$2:J69)</f>
         <v>0.84463386504004478</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L69" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>208</v>
       </c>
@@ -3928,15 +4232,19 @@
         <v>45</v>
       </c>
       <c r="J70" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.5645967236185234E-3</v>
       </c>
       <c r="K70" s="4">
         <f>SUM($J$2:J70)</f>
         <v>0.85019846176366332</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L70" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>212</v>
       </c>
@@ -3965,15 +4273,19 @@
         <v>20</v>
       </c>
       <c r="J71" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.2897738909683228E-3</v>
       </c>
       <c r="K71" s="4">
         <f>SUM($J$2:J71)</f>
         <v>0.85548823565463161</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L71" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -4002,15 +4314,19 @@
         <v>30</v>
       </c>
       <c r="J72" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.2867172233107777E-3</v>
       </c>
       <c r="K72" s="4">
         <f>SUM($J$2:J72)</f>
         <v>0.86077495287794237</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L72" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>104</v>
       </c>
@@ -4039,15 +4355,19 @@
         <v>30</v>
       </c>
       <c r="J73" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.2444099307606589E-3</v>
       </c>
       <c r="K73" s="4">
         <f>SUM($J$2:J73)</f>
         <v>0.86601936280870306</v>
       </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L73" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>200</v>
       </c>
@@ -4076,15 +4396,19 @@
         <v>30</v>
       </c>
       <c r="J74" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>5.063429875825187E-3</v>
       </c>
       <c r="K74" s="4">
         <f>SUM($J$2:J74)</f>
         <v>0.87108279268452826</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L74" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>49</v>
       </c>
@@ -4113,15 +4437,19 @@
         <v>25</v>
       </c>
       <c r="J75" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4.8145562005230801E-3</v>
       </c>
       <c r="K75" s="4">
         <f>SUM($J$2:J75)</f>
         <v>0.87589734888505133</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L75" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>144</v>
       </c>
@@ -4150,15 +4478,19 @@
         <v>25</v>
       </c>
       <c r="J76" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4.8109450198078399E-3</v>
       </c>
       <c r="K76" s="4">
         <f>SUM($J$2:J76)</f>
         <v>0.88070829390485916</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L76" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>118</v>
       </c>
@@ -4187,15 +4519,19 @@
         <v>25</v>
       </c>
       <c r="J77" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4.4254317966652646E-3</v>
       </c>
       <c r="K77" s="4">
         <f>SUM($J$2:J77)</f>
         <v>0.88513372570152438</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L77" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -4224,15 +4560,19 @@
         <v>14</v>
       </c>
       <c r="J78" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4.3407966740443716E-3</v>
       </c>
       <c r="K78" s="4">
         <f>SUM($J$2:J78)</f>
         <v>0.88947452237556879</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L78" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>194</v>
       </c>
@@ -4261,15 +4601,19 @@
         <v>20</v>
       </c>
       <c r="J79" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>4.0124222562852212E-3</v>
       </c>
       <c r="K79" s="4">
         <f>SUM($J$2:J79)</f>
         <v>0.89348694463185396</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L79" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>178</v>
       </c>
@@ -4298,15 +4642,19 @@
         <v>20</v>
       </c>
       <c r="J80" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.9373370807690884E-3</v>
       </c>
       <c r="K80" s="4">
         <f>SUM($J$2:J80)</f>
         <v>0.89742428171262301</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L80" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>116</v>
       </c>
@@ -4335,15 +4683,19 @@
         <v>25</v>
       </c>
       <c r="J81" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.8977783930666835E-3</v>
       </c>
       <c r="K81" s="4">
         <f>SUM($J$2:J81)</f>
         <v>0.90132206010568972</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L81" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>264</v>
       </c>
@@ -4372,15 +4724,19 @@
         <v>20</v>
       </c>
       <c r="J82" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.8110758266998142E-3</v>
       </c>
       <c r="K82" s="4">
         <f>SUM($J$2:J82)</f>
         <v>0.90513313593238953</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L82" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>162</v>
       </c>
@@ -4409,15 +4765,19 @@
         <v>45</v>
       </c>
       <c r="J83" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.8054143168391426E-3</v>
       </c>
       <c r="K83" s="4">
         <f>SUM($J$2:J83)</f>
         <v>0.90893855024922865</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L83" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>218</v>
       </c>
@@ -4446,15 +4806,19 @@
         <v>45</v>
       </c>
       <c r="J84" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.7440037071593949E-3</v>
       </c>
       <c r="K84" s="4">
         <f>SUM($J$2:J84)</f>
         <v>0.91268255395638809</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L84" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>56</v>
       </c>
@@ -4483,15 +4847,19 @@
         <v>30</v>
       </c>
       <c r="J85" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.6335529210746675E-3</v>
       </c>
       <c r="K85" s="4">
         <f>SUM($J$2:J85)</f>
         <v>0.91631610687746279</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L85" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>130</v>
       </c>
@@ -4520,15 +4888,19 @@
         <v>20</v>
       </c>
       <c r="J86" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.6136417947992597E-3</v>
       </c>
       <c r="K86" s="4">
         <f>SUM($J$2:J86)</f>
         <v>0.91992974867226207</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L86" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>184</v>
       </c>
@@ -4557,15 +4929,19 @@
         <v>45</v>
       </c>
       <c r="J87" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.551317265450347E-3</v>
       </c>
       <c r="K87" s="4">
         <f>SUM($J$2:J87)</f>
         <v>0.9234810659377124</v>
       </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L87" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -4594,15 +4970,19 @@
         <v>25</v>
       </c>
       <c r="J88" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.4633447957229517E-3</v>
       </c>
       <c r="K88" s="4">
         <f>SUM($J$2:J88)</f>
         <v>0.92694441073343536</v>
       </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L88" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>166</v>
       </c>
@@ -4631,15 +5011,19 @@
         <v>25</v>
       </c>
       <c r="J89" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.4434473611279809E-3</v>
       </c>
       <c r="K89" s="4">
         <f>SUM($J$2:J89)</f>
         <v>0.93038785809456337</v>
       </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L89" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>170</v>
       </c>
@@ -4668,15 +5052,19 @@
         <v>45</v>
       </c>
       <c r="J90" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.4145681841663829E-3</v>
       </c>
       <c r="K90" s="4">
         <f>SUM($J$2:J90)</f>
         <v>0.93380242627872978</v>
       </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L90" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>64</v>
       </c>
@@ -4705,15 +5093,19 @@
         <v>25</v>
       </c>
       <c r="J91" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.3273692943836743E-3</v>
       </c>
       <c r="K91" s="4">
         <f>SUM($J$2:J91)</f>
         <v>0.93712979557311349</v>
       </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L91" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>98</v>
       </c>
@@ -4742,15 +5134,19 @@
         <v>20</v>
       </c>
       <c r="J92" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.2946153718584246E-3</v>
       </c>
       <c r="K92" s="4">
         <f>SUM($J$2:J92)</f>
         <v>0.94042441094497187</v>
       </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L92" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>156</v>
       </c>
@@ -4779,15 +5175,19 @@
         <v>14</v>
       </c>
       <c r="J93" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>3.2460509813486281E-3</v>
       </c>
       <c r="K93" s="4">
         <f>SUM($J$2:J93)</f>
         <v>0.94367046192632054</v>
       </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L93" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>40</v>
       </c>
@@ -4816,15 +5216,19 @@
         <v>30</v>
       </c>
       <c r="J94" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.9853271566283573E-3</v>
       </c>
       <c r="K94" s="4">
         <f>SUM($J$2:J94)</f>
         <v>0.9466557890829489</v>
       </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L94" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>126</v>
       </c>
@@ -4853,15 +5257,19 @@
         <v>25</v>
       </c>
       <c r="J95" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.9061618603420185E-3</v>
       </c>
       <c r="K95" s="4">
         <f>SUM($J$2:J95)</f>
         <v>0.94956195094329088</v>
       </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L95" t="str">
+        <f t="shared" si="5"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>146</v>
       </c>
@@ -4890,15 +5298,19 @@
         <v>25</v>
       </c>
       <c r="J96" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.9016572974782679E-3</v>
       </c>
       <c r="K96" s="4">
         <f>SUM($J$2:J96)</f>
         <v>0.95246360824076914</v>
       </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L96" t="str">
+        <f t="shared" si="5"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>254</v>
       </c>
@@ -4927,15 +5339,19 @@
         <v>25</v>
       </c>
       <c r="J97" s="7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>2.9006167297650613E-3</v>
       </c>
       <c r="K97" s="4">
         <f>SUM($J$2:J97)</f>
         <v>0.95536422497053419</v>
       </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L97" t="str">
+        <f t="shared" si="5"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>230</v>
       </c>
@@ -4964,15 +5380,19 @@
         <v>45</v>
       </c>
       <c r="J98" s="7">
-        <f t="shared" ref="J98:J121" si="3">F98/SUM($F$2:$F$121)</f>
+        <f t="shared" ref="J98:J121" si="6">F98/SUM($F$2:$F$121)</f>
         <v>2.8784498991376688E-3</v>
       </c>
       <c r="K98" s="4">
         <f>SUM($J$2:J98)</f>
         <v>0.95824267486967185</v>
       </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L98" t="str">
+        <f t="shared" ref="L98:L129" si="7">IF(K98&lt;=80%,"A",IF(K98&lt;=95%,"B","C"))</f>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>262</v>
       </c>
@@ -5001,15 +5421,19 @@
         <v>30</v>
       </c>
       <c r="J99" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.8489272131955348E-3</v>
       </c>
       <c r="K99" s="4">
         <f>SUM($J$2:J99)</f>
         <v>0.96109160208286737</v>
       </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L99" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>138</v>
       </c>
@@ -5038,15 +5462,19 @@
         <v>45</v>
       </c>
       <c r="J100" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.6698160726397044E-3</v>
       </c>
       <c r="K100" s="4">
         <f>SUM($J$2:J100)</f>
         <v>0.96376141815550709</v>
       </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L100" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>174</v>
       </c>
@@ -5075,15 +5503,19 @@
         <v>30</v>
       </c>
       <c r="J101" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.4192617435639645E-3</v>
       </c>
       <c r="K101" s="4">
         <f>SUM($J$2:J101)</f>
         <v>0.96618067989907108</v>
       </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L101" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>122</v>
       </c>
@@ -5112,15 +5544,19 @@
         <v>45</v>
       </c>
       <c r="J102" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.3683629215396711E-3</v>
       </c>
       <c r="K102" s="4">
         <f>SUM($J$2:J102)</f>
         <v>0.96854904282061072</v>
       </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L102" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>232</v>
       </c>
@@ -5149,15 +5585,19 @@
         <v>45</v>
       </c>
       <c r="J103" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.2587370592012687E-3</v>
       </c>
       <c r="K103" s="4">
         <f>SUM($J$2:J103)</f>
         <v>0.97080777987981204</v>
       </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L103" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>124</v>
       </c>
@@ -5186,15 +5626,19 @@
         <v>20</v>
       </c>
       <c r="J104" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.2333629524315252E-3</v>
       </c>
       <c r="K104" s="4">
         <f>SUM($J$2:J104)</f>
         <v>0.97304114283224352</v>
       </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L104" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>244</v>
       </c>
@@ -5223,15 +5667,19 @@
         <v>30</v>
       </c>
       <c r="J105" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.2299913761239308E-3</v>
       </c>
       <c r="K105" s="4">
         <f>SUM($J$2:J105)</f>
         <v>0.97527113420836742</v>
       </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L105" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>82</v>
       </c>
@@ -5260,15 +5708,19 @@
         <v>25</v>
       </c>
       <c r="J106" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.2238369657675301E-3</v>
       </c>
       <c r="K106" s="4">
         <f>SUM($J$2:J106)</f>
         <v>0.97749497117413497</v>
       </c>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L106" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>270</v>
       </c>
@@ -5297,15 +5749,19 @@
         <v>30</v>
       </c>
       <c r="J107" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.1583565040779046E-3</v>
       </c>
       <c r="K107" s="4">
         <f>SUM($J$2:J107)</f>
         <v>0.97965332767821289</v>
       </c>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L107" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>222</v>
       </c>
@@ -5334,15 +5790,19 @@
         <v>20</v>
       </c>
       <c r="J108" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.1346664740019036E-3</v>
       </c>
       <c r="K108" s="4">
         <f>SUM($J$2:J108)</f>
         <v>0.98178799415221485</v>
       </c>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L108" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>66</v>
       </c>
@@ -5371,15 +5831,19 @@
         <v>45</v>
       </c>
       <c r="J109" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.8591111364483265E-3</v>
       </c>
       <c r="K109" s="4">
         <f>SUM($J$2:J109)</f>
         <v>0.98364710528866317</v>
       </c>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L109" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>160</v>
       </c>
@@ -5408,15 +5872,19 @@
         <v>30</v>
       </c>
       <c r="J110" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.8322651740316127E-3</v>
       </c>
       <c r="K110" s="4">
         <f>SUM($J$2:J110)</f>
         <v>0.98547937046269474</v>
       </c>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L110" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>240</v>
       </c>
@@ -5445,15 +5913,19 @@
         <v>30</v>
       </c>
       <c r="J111" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.7383881671157908E-3</v>
       </c>
       <c r="K111" s="4">
         <f>SUM($J$2:J111)</f>
         <v>0.98721775862981054</v>
       </c>
-    </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L111" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>242</v>
       </c>
@@ -5482,15 +5954,19 @@
         <v>45</v>
       </c>
       <c r="J112" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.4586568670289497E-3</v>
       </c>
       <c r="K112" s="4">
         <f>SUM($J$2:J112)</f>
         <v>0.98867641549683949</v>
       </c>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L112" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>31</v>
       </c>
@@ -5519,15 +5995,19 @@
         <v>25</v>
       </c>
       <c r="J113" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.4389921910014066E-3</v>
       </c>
       <c r="K113" s="4">
         <f>SUM($J$2:J113)</f>
         <v>0.9901154076878409</v>
       </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L113" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>112</v>
       </c>
@@ -5556,15 +6036,19 @@
         <v>45</v>
       </c>
       <c r="J114" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.421525029683991E-3</v>
       </c>
       <c r="K114" s="4">
         <f>SUM($J$2:J114)</f>
         <v>0.99153693271752485</v>
       </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L114" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>224</v>
       </c>
@@ -5593,15 +6077,19 @@
         <v>25</v>
       </c>
       <c r="J115" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.3989577174038186E-3</v>
       </c>
       <c r="K115" s="4">
         <f>SUM($J$2:J115)</f>
         <v>0.99293589043492869</v>
       </c>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L115" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>142</v>
       </c>
@@ -5630,15 +6118,19 @@
         <v>20</v>
       </c>
       <c r="J116" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.3776534626439528E-3</v>
       </c>
       <c r="K116" s="4">
         <f>SUM($J$2:J116)</f>
         <v>0.99431354389757265</v>
       </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L116" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>37</v>
       </c>
@@ -5667,15 +6159,19 @@
         <v>20</v>
       </c>
       <c r="J117" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.3374238826001385E-3</v>
       </c>
       <c r="K117" s="4">
         <f>SUM($J$2:J117)</f>
         <v>0.99565096778017281</v>
       </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L117" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>248</v>
       </c>
@@ -5704,15 +6200,19 @@
         <v>30</v>
       </c>
       <c r="J118" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.3267409489392224E-3</v>
       </c>
       <c r="K118" s="4">
         <f>SUM($J$2:J118)</f>
         <v>0.99697770872911207</v>
       </c>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L118" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>256</v>
       </c>
@@ -5741,15 +6241,19 @@
         <v>25</v>
       </c>
       <c r="J119" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.1036384391395306E-3</v>
       </c>
       <c r="K119" s="4">
         <f>SUM($J$2:J119)</f>
         <v>0.99808134716825159</v>
       </c>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L119" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>140</v>
       </c>
@@ -5778,15 +6282,19 @@
         <v>45</v>
       </c>
       <c r="J120" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>9.8864886098996027E-4</v>
       </c>
       <c r="K120" s="4">
         <f>SUM($J$2:J120)</f>
         <v>0.99906999602924151</v>
       </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L120" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>182</v>
       </c>
@@ -5815,12 +6323,16 @@
         <v>30</v>
       </c>
       <c r="J121" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>9.3000397075847273E-4</v>
       </c>
       <c r="K121" s="4">
         <f>SUM($J$2:J121)</f>
         <v>1</v>
+      </c>
+      <c r="L121" t="str">
+        <f t="shared" si="7"/>
+        <v>C</v>
       </c>
     </row>
   </sheetData>
@@ -5832,6 +6344,60 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD49C0F8-9F96-4F47-B62A-6FDD67704BE5}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>297</v>
+      </c>
+      <c r="B1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2">
+        <f>COUNTIF(Suppliers!L:L,A2)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>300</v>
+      </c>
+      <c r="B3">
+        <f>COUNTIF(Suppliers!L:L,A3)</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>301</v>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(Suppliers!L:L,A4)</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>302</v>
+      </c>
+      <c r="B5">
+        <f>SUM(B2:B4)</f>
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -5933,7 +6499,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
M6 step 3a: empty PivotTable on Results sheet (fields still to add); other workbooks re-saved in Excel
</commit_message>
<xml_diff>
--- a/excel/Spend_Analysis.xlsx
+++ b/excel/Spend_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B97F94-08BF-8B4F-BA3C-1F4F66E5B685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F721CC40-A1A4-8F42-88B2-EF619393B6DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +19,9 @@
     <sheet name="Settings" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="3" r:id="rId5"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -997,7 +1000,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1005,12 +1008,123 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1021,6 +1135,15 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1044,6 +1167,1771 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="mac" refreshedDate="46304.91306111111" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="120" xr:uid="{1DF923C8-D7D4-D946-94B0-EB1C7771341B}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="tblSpend"/>
+  </cacheSource>
+  <cacheFields count="12">
+    <cacheField name="Golden ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Supplier" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Country" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Commodity" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Segment (M2)" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Spend (EUR)" numFmtId="3">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="271699" maxValue="8729465"/>
+    </cacheField>
+    <cacheField name="OTD %" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="16.7" maxValue="100"/>
+    </cacheField>
+    <cacheField name="PPM" numFmtId="3">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="5338"/>
+    </cacheField>
+    <cacheField name="Payment term" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Spend share" numFmtId="9">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="9.3000397075847273E-4" maxValue="2.9880261291344874E-2"/>
+    </cacheField>
+    <cacheField name="Cumulative share" numFmtId="9">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.9880261291344874E-2" maxValue="1"/>
+    </cacheField>
+    <cacheField name="ABC class" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="120">
+  <r>
+    <s v="G0098"/>
+    <s v="KAPPATEC GMBH"/>
+    <s v="AT"/>
+    <s v="Plastic housings"/>
+    <s v="Strategic and reliable"/>
+    <n v="8729465"/>
+    <n v="87"/>
+    <n v="117"/>
+    <s v="NT60"/>
+    <n v="2.9880261291344874E-2"/>
+    <n v="2.9880261291344874E-2"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0016"/>
+    <s v="Lumencast GmbH"/>
+    <s v="AT"/>
+    <s v="Packaging"/>
+    <s v="Quality risk"/>
+    <n v="8166335"/>
+    <n v="94.9"/>
+    <n v="699"/>
+    <s v="missing"/>
+    <n v="2.7952712290232544E-2"/>
+    <n v="5.7832973581577421E-2"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0102"/>
+    <s v="Deltaarts SAS"/>
+    <s v="FR"/>
+    <s v="Valves"/>
+    <s v="Strategic and reliable"/>
+    <n v="7892755"/>
+    <n v="93.3"/>
+    <n v="134"/>
+    <s v="NT30"/>
+    <n v="2.7016269806748604E-2"/>
+    <n v="8.4849243388326029E-2"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0052"/>
+    <s v="Krafttec GmbH"/>
+    <s v="DE"/>
+    <s v="Plastic housings"/>
+    <s v="Quality risk"/>
+    <n v="7297508"/>
+    <n v="85.1"/>
+    <n v="789"/>
+    <s v="NT60"/>
+    <n v="2.4978786880488043E-2"/>
+    <n v="0.10982803026881408"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0012"/>
+    <s v="Velawerk s.r.o."/>
+    <s v="CZ"/>
+    <s v="Plastic housings"/>
+    <s v="Strategic and reliable"/>
+    <n v="7016505"/>
+    <n v="96.3"/>
+    <n v="102"/>
+    <s v="NT45"/>
+    <n v="2.4016936061033268E-2"/>
+    <n v="0.13384496632984735"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0083"/>
+    <s v="Kappawerk GmbH"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Strategic and reliable"/>
+    <n v="6591040"/>
+    <n v="92.4"/>
+    <n v="117"/>
+    <s v="NT30"/>
+    <n v="2.2560603356758486E-2"/>
+    <n v="0.15640556968660585"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0103"/>
+    <s v="TAUROGUSS GMBH"/>
+    <s v="DE"/>
+    <s v="Rubber seals"/>
+    <s v="Strategic and reliable"/>
+    <n v="6508860"/>
+    <n v="88.2"/>
+    <n v="60"/>
+    <s v="SK14"/>
+    <n v="2.2279307782181727E-2"/>
+    <n v="0.17868487746878758"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0044"/>
+    <s v="Ventoplast GmbH"/>
+    <s v="DE"/>
+    <s v="Electronic sensors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="6491982"/>
+    <n v="58.8"/>
+    <n v="911"/>
+    <s v="NT60"/>
+    <n v="2.2221535736578094E-2"/>
+    <n v="0.20090641320536567"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0063"/>
+    <s v="Polarcast Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Valves"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="6425100"/>
+    <n v="79.3"/>
+    <n v="5265"/>
+    <s v="NT45"/>
+    <n v="2.1992603993832377E-2"/>
+    <n v="0.22289901719919805"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0094"/>
+    <s v="Cerroparts"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Strategic and reliable"/>
+    <n v="6072516"/>
+    <n v="96.5"/>
+    <n v="104"/>
+    <s v="NT60"/>
+    <n v="2.07857371300386E-2"/>
+    <n v="0.24368475432923664"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0077"/>
+    <s v="Orbisparts GmbH"/>
+    <s v="DE"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="5969282"/>
+    <n v="64.099999999999994"/>
+    <n v="916"/>
+    <s v="NT45"/>
+    <n v="2.0432375395482049E-2"/>
+    <n v="0.26411712972471868"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0117"/>
+    <s v="Deltaflex  Sp.  z  o.o."/>
+    <s v="PL"/>
+    <s v="Aluminium castings"/>
+    <s v="Delivery risk"/>
+    <n v="5915328"/>
+    <n v="51.6"/>
+    <n v="114"/>
+    <s v="NT60"/>
+    <n v="2.0247695163908497E-2"/>
+    <n v="0.28436482488862719"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0087"/>
+    <s v="Polarplast  S.r.l."/>
+    <s v="IT"/>
+    <s v="Valves"/>
+    <s v="Strategic and reliable"/>
+    <n v="5803633"/>
+    <n v="88.9"/>
+    <n v="50"/>
+    <s v="SK14"/>
+    <n v="1.9865372102307727E-2"/>
+    <n v="0.3042301969909349"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0074"/>
+    <s v="Alpenguss SAS"/>
+    <s v="FR"/>
+    <s v="Fasteners"/>
+    <s v="Quality risk"/>
+    <n v="5528859"/>
+    <n v="90.4"/>
+    <n v="806"/>
+    <s v="NT30"/>
+    <n v="1.8924842652213364E-2"/>
+    <n v="0.32315503964314829"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0114"/>
+    <s v="Orbisflex GmbH"/>
+    <s v="DE"/>
+    <s v="Plastic housings"/>
+    <s v="Delivery risk"/>
+    <n v="4891366"/>
+    <n v="83.1"/>
+    <n v="140"/>
+    <s v="NT60"/>
+    <n v="1.6742755043018146E-2"/>
+    <n v="0.33989779468616643"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0070"/>
+    <s v="Terraparts GmbH"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Delivery risk"/>
+    <n v="4886318"/>
+    <n v="67.900000000000006"/>
+    <n v="173"/>
+    <s v="NT30"/>
+    <n v="1.6725476142306739E-2"/>
+    <n v="0.35662327082847317"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0022"/>
+    <s v="Velacast GmbH"/>
+    <s v="AT"/>
+    <s v="Plastic housings"/>
+    <s v="Strategic and reliable"/>
+    <n v="4635149"/>
+    <n v="91.8"/>
+    <n v="24"/>
+    <s v="NT60"/>
+    <n v="1.586574472139082E-2"/>
+    <n v="0.37248901554986397"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0009"/>
+    <s v="Alpentronic GmbH"/>
+    <s v="DE"/>
+    <s v="Rubber seals"/>
+    <s v="Strategic and reliable"/>
+    <n v="4527145"/>
+    <n v="96.6"/>
+    <n v="75"/>
+    <s v="NT45"/>
+    <n v="1.5496055657913227E-2"/>
+    <n v="0.3879850712077772"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0048"/>
+    <s v="Ferrocast GmbH"/>
+    <s v="DE"/>
+    <s v="Aluminium castings"/>
+    <s v="Quality risk"/>
+    <n v="4516419"/>
+    <n v="94.1"/>
+    <n v="747"/>
+    <s v="NT45"/>
+    <n v="1.5459341416821594E-2"/>
+    <n v="0.40344441262459879"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0058"/>
+    <s v="Boraline GmbH"/>
+    <s v="DE"/>
+    <s v="Fasteners"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="4112508"/>
+    <n v="41.7"/>
+    <n v="980"/>
+    <s v="NT60"/>
+    <n v="1.407678633258122E-2"/>
+    <n v="0.41752119895717998"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0080"/>
+    <s v="Velaline S.r.l."/>
+    <s v="IT"/>
+    <s v="Aluminium castings"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="4009816"/>
+    <n v="73.8"/>
+    <n v="893"/>
+    <s v="NT60"/>
+    <n v="1.3725279820723874E-2"/>
+    <n v="0.43124647877790384"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0082"/>
+    <s v="Ferrotronic S.r.l."/>
+    <s v="IT"/>
+    <s v="Plastic housings"/>
+    <s v="Delivery risk"/>
+    <n v="3901204"/>
+    <n v="70"/>
+    <n v="146"/>
+    <s v="NT60"/>
+    <n v="1.3353509621819869E-2"/>
+    <n v="0.4445999883997237"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0002"/>
+    <s v="Ferroform s.r.o."/>
+    <s v="CZ"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="3850896"/>
+    <n v="77.099999999999994"/>
+    <n v="902"/>
+    <s v="NT60"/>
+    <n v="1.318130935696458E-2"/>
+    <n v="0.4577812977566883"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0101"/>
+    <s v="RHEINGUSS SAS"/>
+    <s v="FR"/>
+    <s v="Plastic housings"/>
+    <s v="Delivery risk"/>
+    <n v="3790329"/>
+    <n v="58.8"/>
+    <n v="164"/>
+    <s v="NT30"/>
+    <n v="1.297399335470867E-2"/>
+    <n v="0.47075529111139697"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0118"/>
+    <s v="Cerroform  S.r.l."/>
+    <s v="IT"/>
+    <s v="Valves"/>
+    <s v="Strategic and reliable"/>
+    <n v="3669523"/>
+    <n v="95.9"/>
+    <n v="90"/>
+    <s v="NT30"/>
+    <n v="1.2560484067992679E-2"/>
+    <n v="0.48331577517938967"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0079"/>
+    <s v="Primaparts GmbH"/>
+    <s v="DE"/>
+    <s v="Electronic sensors"/>
+    <s v="Strategic and reliable"/>
+    <n v="3559963"/>
+    <n v="90"/>
+    <n v="87"/>
+    <s v="NT30"/>
+    <n v="1.2185468940825122E-2"/>
+    <n v="0.49550124412021479"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0024"/>
+    <s v="NORDCAST SP. Z O.O."/>
+    <s v="PL"/>
+    <s v="Plastic housings"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="3489820"/>
+    <n v="82.1"/>
+    <n v="743"/>
+    <s v="SK14"/>
+    <n v="1.1945375055603199E-2"/>
+    <n v="0.50744661917581801"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0032"/>
+    <s v="Voltacast GmbH"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Quality risk"/>
+    <n v="3460790"/>
+    <n v="94.9"/>
+    <n v="797"/>
+    <s v="NT45"/>
+    <n v="1.1846007684832167E-2"/>
+    <n v="0.51929262686065014"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0085"/>
+    <s v="Voltatec GmbH"/>
+    <s v="DE"/>
+    <s v="Aluminium castings"/>
+    <s v="Quality risk"/>
+    <n v="3429954"/>
+    <n v="86.5"/>
+    <n v="5270"/>
+    <s v="SK14"/>
+    <n v="1.1740458520343861E-2"/>
+    <n v="0.53103308538099403"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0038"/>
+    <s v="Voltawerk GmbH"/>
+    <s v="DE"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="3295628"/>
+    <n v="65.5"/>
+    <n v="943"/>
+    <s v="NT60"/>
+    <n v="1.128067135375104E-2"/>
+    <n v="0.54231375673474502"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0037"/>
+    <s v="Ferroflex GmbH"/>
+    <s v="DE"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="3104710"/>
+    <n v="72.5"/>
+    <n v="748"/>
+    <s v="NT30"/>
+    <n v="1.0627174292336512E-2"/>
+    <n v="0.55294093102708153"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0086"/>
+    <s v="Terraseal  SAS"/>
+    <s v="FR"/>
+    <s v="Rubber seals"/>
+    <s v="Strategic and reliable"/>
+    <n v="3090622"/>
+    <n v="94.1"/>
+    <n v="133"/>
+    <s v="SK14"/>
+    <n v="1.0578952193837638E-2"/>
+    <n v="0.56351988322091917"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0028"/>
+    <s v="Novaseal GmbH"/>
+    <s v="DE"/>
+    <s v="Rubber seals"/>
+    <s v="Quality risk"/>
+    <n v="3030493"/>
+    <n v="91.9"/>
+    <n v="835"/>
+    <s v="SK14"/>
+    <n v="1.0373135430589573E-2"/>
+    <n v="0.57389301865150877"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0015"/>
+    <s v="Silberline S.r.l."/>
+    <s v="IT"/>
+    <s v="Packaging"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="2959201"/>
+    <n v="54.3"/>
+    <n v="670"/>
+    <s v="SK14"/>
+    <n v="1.0129108610162139E-2"/>
+    <n v="0.58402212726167091"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0006"/>
+    <s v="Aquametal GmbH"/>
+    <s v="DE"/>
+    <s v="Valves"/>
+    <s v="Delivery risk"/>
+    <n v="2943032"/>
+    <n v="75"/>
+    <n v="85"/>
+    <s v="NT60"/>
+    <n v="1.0073763414915953E-2"/>
+    <n v="0.59409589067658686"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0091"/>
+    <s v="Nordplast  s.r.o."/>
+    <s v="CZ"/>
+    <s v="Rubber seals"/>
+    <s v="Delivery risk"/>
+    <n v="2923417"/>
+    <n v="42.5"/>
+    <n v="127"/>
+    <s v="SK14"/>
+    <n v="1.000662283697335E-2"/>
+    <n v="0.60410251351356026"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0004"/>
+    <s v="Ventoline S.r.l."/>
+    <s v="IT"/>
+    <s v="Electronic sensors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="2882552"/>
+    <n v="81.8"/>
+    <n v="869"/>
+    <s v="NT30"/>
+    <n v="9.8667452067095467E-3"/>
+    <n v="0.61396925872026975"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0023"/>
+    <s v="Taurometal Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="2871672"/>
+    <n v="76.5"/>
+    <n v="4588"/>
+    <s v="NT30"/>
+    <n v="9.8295038359210926E-3"/>
+    <n v="0.62379876255619082"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0059"/>
+    <s v="Alpencast Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Delivery risk"/>
+    <n v="2865400"/>
+    <n v="64.5"/>
+    <n v="19"/>
+    <s v="SK14"/>
+    <n v="9.8080352809959831E-3"/>
+    <n v="0.63360679783718676"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0026"/>
+    <s v="Kappaplast GmbH"/>
+    <s v="DE"/>
+    <s v="Fasteners"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="2825038"/>
+    <n v="73.099999999999994"/>
+    <n v="816"/>
+    <s v="NT60"/>
+    <n v="9.6698793795471239E-3"/>
+    <n v="0.64327667721673387"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0050"/>
+    <s v="Atlasflex GmbH"/>
+    <s v="AT"/>
+    <s v="Electronic sensors"/>
+    <s v="Strategic and reliable"/>
+    <n v="2697901"/>
+    <n v="96.9"/>
+    <n v="113"/>
+    <s v="NT30"/>
+    <n v="9.2346995856195796E-3"/>
+    <n v="0.65251137680235349"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0061"/>
+    <s v="Kraftflex s.r.o."/>
+    <s v="CZ"/>
+    <s v="Plastic housings"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="2629295"/>
+    <n v="36.4"/>
+    <n v="863"/>
+    <s v="NT60"/>
+    <n v="8.9998667286055462E-3"/>
+    <n v="0.66151124353095903"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0030"/>
+    <s v="Silbermetal s.r.o."/>
+    <s v="CZ"/>
+    <s v="Valves"/>
+    <s v="Strategic and reliable"/>
+    <n v="2483150"/>
+    <n v="90.9"/>
+    <n v="68"/>
+    <s v="NT60"/>
+    <n v="8.4996240692417034E-3"/>
+    <n v="0.67001086760020068"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0010"/>
+    <s v="Deltaguss GmbH"/>
+    <s v="DE"/>
+    <s v="Fasteners"/>
+    <s v="Delivery risk"/>
+    <n v="2466796"/>
+    <n v="51.6"/>
+    <n v="68"/>
+    <s v="NT45"/>
+    <n v="8.4436456337753079E-3"/>
+    <n v="0.67845451323397599"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0035"/>
+    <s v="Alpenwerk GmbH"/>
+    <s v="AT"/>
+    <s v="Electronic sensors"/>
+    <s v="Quality risk"/>
+    <n v="2435186"/>
+    <n v="96"/>
+    <n v="4612"/>
+    <s v="NT30"/>
+    <n v="8.3354471291224551E-3"/>
+    <n v="0.68678996036309847"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0113"/>
+    <s v="FERROMETAL GMBH"/>
+    <s v="DE"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Strategic and reliable"/>
+    <n v="2325849"/>
+    <n v="90"/>
+    <n v="189"/>
+    <s v="NT45"/>
+    <n v="7.9611953131392566E-3"/>
+    <n v="0.69475115567623769"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0039"/>
+    <s v="Ferroparts GmbH"/>
+    <s v="DE"/>
+    <s v="Electronic sensors"/>
+    <s v="Strategic and reliable"/>
+    <n v="2314507"/>
+    <n v="93.9"/>
+    <n v="110"/>
+    <s v="NT60"/>
+    <n v="7.9223725532603373E-3"/>
+    <n v="0.70267352822949802"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0051"/>
+    <s v="Voltaplast GmbH"/>
+    <s v="DE"/>
+    <s v="Fasteners"/>
+    <s v="Delivery risk"/>
+    <n v="2304631"/>
+    <n v="71.400000000000006"/>
+    <n v="100"/>
+    <s v="missing"/>
+    <n v="7.8885677942615532E-3"/>
+    <n v="0.71056209602375953"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0031"/>
+    <s v="Kraftseal S.r.l."/>
+    <s v="IT"/>
+    <s v="Valves"/>
+    <s v="Strategic and reliable"/>
+    <n v="2255266"/>
+    <n v="85.7"/>
+    <n v="134"/>
+    <s v="NT60"/>
+    <n v="7.7195953430692701E-3"/>
+    <n v="0.71828169136682884"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0021"/>
+    <s v="Velaguss Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Plastic housings"/>
+    <s v="Delivery risk"/>
+    <n v="2235309"/>
+    <n v="65"/>
+    <n v="76"/>
+    <s v="NT45"/>
+    <n v="7.6512841264493089E-3"/>
+    <n v="0.72593297549327818"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0041"/>
+    <s v="Atlasplast Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Strategic and reliable"/>
+    <n v="2128201"/>
+    <n v="100"/>
+    <n v="109"/>
+    <s v="NT30"/>
+    <n v="7.2846619993895906E-3"/>
+    <n v="0.73321763749266777"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0027"/>
+    <s v="PRIMAFORM S.R.L."/>
+    <s v="IT"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Strategic and reliable"/>
+    <n v="2119288"/>
+    <n v="91.7"/>
+    <n v="147"/>
+    <s v="NT60"/>
+    <n v="7.2541535124559979E-3"/>
+    <n v="0.74047179100512373"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0109"/>
+    <s v="Vltatronic Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Valves"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="2096576"/>
+    <n v="72.2"/>
+    <n v="1167"/>
+    <s v="NT60"/>
+    <n v="7.1764121509350996E-3"/>
+    <n v="0.74764820315605884"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0097"/>
+    <s v="Kraftcast  Sp.  z  o.o."/>
+    <s v="PL"/>
+    <s v="Electronic sensors"/>
+    <s v="Strategic and reliable"/>
+    <n v="2078432"/>
+    <n v="94.6"/>
+    <n v="167"/>
+    <s v="NT30"/>
+    <n v="7.1143066884731777E-3"/>
+    <n v="0.75476250984453197"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0120"/>
+    <s v="Taurotec  GmbH"/>
+    <s v="DE"/>
+    <s v="Aluminium castings"/>
+    <s v="Strategic and reliable"/>
+    <n v="2056747"/>
+    <n v="94.7"/>
+    <n v="107"/>
+    <s v="SK14"/>
+    <n v="7.0400806659044624E-3"/>
+    <n v="0.76180259051043642"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0072"/>
+    <s v="Nordwerk GmbH"/>
+    <s v="AT"/>
+    <s v="Rubber seals"/>
+    <s v="Quality risk"/>
+    <n v="2053464"/>
+    <n v="87.5"/>
+    <n v="1013"/>
+    <s v="NT45"/>
+    <n v="7.0288432191858508E-3"/>
+    <n v="0.76883143372962226"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0110"/>
+    <s v="KRAFTFORM SAS"/>
+    <s v="FR"/>
+    <s v="Rubber seals"/>
+    <s v="Quality risk"/>
+    <n v="1985456"/>
+    <n v="86.7"/>
+    <n v="730"/>
+    <s v="NT45"/>
+    <n v="6.796057268397139E-3"/>
+    <n v="0.77562749099801942"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0029"/>
+    <s v="Ventoseal GmbH"/>
+    <s v="DE"/>
+    <s v="Valves"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1970618"/>
+    <n v="73.7"/>
+    <n v="718"/>
+    <s v="NT60"/>
+    <n v="6.745267979816341E-3"/>
+    <n v="0.78237275897783576"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0013"/>
+    <s v="Tauroparts S.r.l."/>
+    <s v="IT"/>
+    <s v="Electronic sensors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1919165"/>
+    <n v="72.2"/>
+    <n v="810"/>
+    <s v="NT30"/>
+    <n v="6.56914847143598E-3"/>
+    <n v="0.78894190744927173"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0066"/>
+    <s v="Boratronic SAS"/>
+    <s v="FR"/>
+    <s v="Electronic sensors"/>
+    <s v="Strategic and reliable"/>
+    <n v="1917140"/>
+    <n v="88"/>
+    <n v="109"/>
+    <s v="SK14"/>
+    <n v="6.5622170582147832E-3"/>
+    <n v="0.79550412450748653"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <s v="G0068"/>
+    <s v="Deltametal Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Delivery risk"/>
+    <n v="1878888"/>
+    <n v="68.8"/>
+    <n v="145"/>
+    <s v="NT60"/>
+    <n v="6.4312835181964062E-3"/>
+    <n v="0.80193540802568297"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0034"/>
+    <s v="Novametal Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Reliable, lower spend"/>
+    <n v="1870250"/>
+    <n v="100"/>
+    <n v="0"/>
+    <s v="NT60"/>
+    <n v="6.4017163342928521E-3"/>
+    <n v="0.80833712435997584"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0019"/>
+    <s v="Kraftguss s.r.o."/>
+    <s v="CZ"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1863627"/>
+    <n v="57.1"/>
+    <n v="4508"/>
+    <s v="SK14"/>
+    <n v="6.3790463344094023E-3"/>
+    <n v="0.81471617069438529"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0078"/>
+    <s v="Velaseal s.r.o."/>
+    <s v="CZ"/>
+    <s v="Valves"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1818970"/>
+    <n v="44.4"/>
+    <n v="4723"/>
+    <s v="NT30"/>
+    <n v="6.2261889910913883E-3"/>
+    <n v="0.82094235968547669"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0092"/>
+    <s v="RHEINSEAL GMBH"/>
+    <s v="DE"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Delivery risk"/>
+    <n v="1780307"/>
+    <n v="79.3"/>
+    <n v="135"/>
+    <s v="SK14"/>
+    <n v="6.0938486309081163E-3"/>
+    <n v="0.8270362083163848"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0107"/>
+    <s v="Nordtronic"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Delivery risk"/>
+    <n v="1727420"/>
+    <n v="42.9"/>
+    <n v="165"/>
+    <s v="SK14"/>
+    <n v="5.9128206550911151E-3"/>
+    <n v="0.83294902897147594"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0060"/>
+    <s v="Atlasparts Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Electronic sensors"/>
+    <s v="Reliable, lower spend"/>
+    <n v="1719814"/>
+    <n v="94.1"/>
+    <n v="110"/>
+    <s v="NT60"/>
+    <n v="5.8867859247402898E-3"/>
+    <n v="0.83883581489621628"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0089"/>
+    <s v="Boratc S.r.l."/>
+    <s v="IT"/>
+    <s v="Electronic sensors"/>
+    <s v="Quality risk"/>
+    <n v="1693890"/>
+    <n v="94.7"/>
+    <n v="705"/>
+    <s v="SK14"/>
+    <n v="5.7980501438285358E-3"/>
+    <n v="0.84463386504004478"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0088"/>
+    <s v="Orbisguss"/>
+    <s v="DE"/>
+    <s v="Rubber seals"/>
+    <s v="Delivery risk"/>
+    <n v="1625687"/>
+    <n v="70.599999999999994"/>
+    <n v="211"/>
+    <s v="NT45"/>
+    <n v="5.5645967236185234E-3"/>
+    <n v="0.85019846176366332"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0090"/>
+    <s v="Tauroseal"/>
+    <s v="DE"/>
+    <s v="Aluminium castings"/>
+    <s v="Delivery risk"/>
+    <n v="1545398"/>
+    <n v="54.2"/>
+    <n v="0"/>
+    <s v="NT60"/>
+    <n v="5.2897738909683228E-3"/>
+    <n v="0.85548823565463161"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0020"/>
+    <s v="Boraseal GmbH"/>
+    <s v="DE"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1544505"/>
+    <n v="63.6"/>
+    <n v="861"/>
+    <s v="NT30"/>
+    <n v="5.2867172233107777E-3"/>
+    <n v="0.86077495287794237"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0036"/>
+    <s v="Atlasguss  GmbH"/>
+    <s v="DE"/>
+    <s v="Rubber seals"/>
+    <s v="Reliable, lower spend"/>
+    <n v="1532145"/>
+    <n v="87.5"/>
+    <n v="118"/>
+    <s v="NT30"/>
+    <n v="5.2444099307606589E-3"/>
+    <n v="0.86601936280870306"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0084"/>
+    <s v="Silberwerk s.r.o."/>
+    <s v="CZ"/>
+    <s v="Electronic sensors"/>
+    <s v="Delivery risk"/>
+    <n v="1479272"/>
+    <n v="63.6"/>
+    <n v="53"/>
+    <s v="NT30"/>
+    <n v="5.063429875825187E-3"/>
+    <n v="0.87108279268452826"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0011"/>
+    <s v="Cerrocast s.r.o."/>
+    <s v="CZ"/>
+    <s v="Valves"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1406564"/>
+    <n v="52.2"/>
+    <n v="885"/>
+    <s v="SK14"/>
+    <n v="4.8145562005230801E-3"/>
+    <n v="0.87589734888505133"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0056"/>
+    <s v="Deltaform Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Packaging"/>
+    <s v="Quality risk"/>
+    <n v="1405509"/>
+    <n v="95.2"/>
+    <n v="5227"/>
+    <s v="SK14"/>
+    <n v="4.8109450198078399E-3"/>
+    <n v="0.88070829390485916"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0043"/>
+    <s v="Cerrowerk Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Delivery risk"/>
+    <n v="1292882"/>
+    <n v="57.1"/>
+    <n v="248"/>
+    <s v="SK14"/>
+    <n v="4.4254317966652646E-3"/>
+    <n v="0.88513372570152438"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0001"/>
+    <s v="Deltaplast GmbH"/>
+    <s v="DE"/>
+    <s v="Aluminium castings"/>
+    <s v="Reliable, lower spend"/>
+    <n v="1268156"/>
+    <n v="100"/>
+    <n v="81"/>
+    <s v="missing"/>
+    <n v="4.3407966740443716E-3"/>
+    <n v="0.88947452237556879"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0081"/>
+    <s v="Aquaplast s.r.o."/>
+    <s v="CZ"/>
+    <s v="Rubber seals"/>
+    <s v="Reliable, lower spend"/>
+    <n v="1172222"/>
+    <n v="85.7"/>
+    <n v="75"/>
+    <s v="NT60"/>
+    <n v="4.0124222562852212E-3"/>
+    <n v="0.89348694463185396"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0073"/>
+    <s v="Ventoguss GmbH"/>
+    <s v="DE"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1150286"/>
+    <n v="58.3"/>
+    <n v="1048"/>
+    <s v="NT60"/>
+    <n v="3.9373370807690884E-3"/>
+    <n v="0.89742428171262301"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0042"/>
+    <s v="Tauroform Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Rubber seals"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1138729"/>
+    <n v="46.2"/>
+    <n v="550"/>
+    <s v="SK14"/>
+    <n v="3.8977783930666835E-3"/>
+    <n v="0.90132206010568972"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0116"/>
+    <s v="Atlastronc GmbH"/>
+    <s v="DE"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Reliable, lower spend"/>
+    <n v="1113399"/>
+    <n v="100"/>
+    <n v="288"/>
+    <s v="NT60"/>
+    <n v="3.8110758266998142E-3"/>
+    <n v="0.90513313593238953"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0065"/>
+    <s v="Kappaform GmbH"/>
+    <s v="AT"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Delivery risk"/>
+    <n v="1111745"/>
+    <n v="80"/>
+    <n v="74"/>
+    <s v="NT45"/>
+    <n v="3.8054143168391426E-3"/>
+    <n v="0.90893855024922865"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0093"/>
+    <s v="Orbistronic"/>
+    <s v="IT"/>
+    <s v="Electronic sensors"/>
+    <s v="Delivery risk"/>
+    <n v="1093804"/>
+    <n v="69.2"/>
+    <n v="81"/>
+    <s v="NT45"/>
+    <n v="3.7440037071593949E-3"/>
+    <n v="0.91268255395638809"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0014"/>
+    <s v="Velaparts s.r.o."/>
+    <s v="CZ"/>
+    <s v="Rubber seals"/>
+    <s v="Quality risk"/>
+    <n v="1061536"/>
+    <n v="90.9"/>
+    <n v="503"/>
+    <s v="NT30"/>
+    <n v="3.6335529210746675E-3"/>
+    <n v="0.91631610687746279"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0049"/>
+    <s v="Novaline GmbH"/>
+    <s v="DE"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="1055719"/>
+    <n v="76.900000000000006"/>
+    <n v="725"/>
+    <s v="NT60"/>
+    <n v="3.6136417947992597E-3"/>
+    <n v="0.91992974867226207"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0076"/>
+    <s v="Aquatronic GmbH"/>
+    <s v="DE"/>
+    <s v="Rubber seals"/>
+    <s v="Delivery risk"/>
+    <n v="1037511"/>
+    <n v="70"/>
+    <n v="116"/>
+    <s v="NT45"/>
+    <n v="3.551317265450347E-3"/>
+    <n v="0.9234810659377124"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0003"/>
+    <s v="Atlaswerk GmbH"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Delivery risk"/>
+    <n v="1011810"/>
+    <n v="80"/>
+    <n v="0"/>
+    <s v="SK14"/>
+    <n v="3.4633447957229517E-3"/>
+    <n v="0.92694441073343536"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0067"/>
+    <s v="Polarmetal s.r.o."/>
+    <s v="CZ"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Quality risk"/>
+    <n v="1005997"/>
+    <n v="100"/>
+    <n v="5294"/>
+    <s v="SK14"/>
+    <n v="3.4434473611279809E-3"/>
+    <n v="0.93038785809456337"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0069"/>
+    <s v="Lumenwerk s.r.o."/>
+    <s v="CZ"/>
+    <s v="Plastic housings"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="997560"/>
+    <n v="72.7"/>
+    <n v="1095"/>
+    <s v="NT45"/>
+    <n v="3.4145681841663829E-3"/>
+    <n v="0.93380242627872978"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0017"/>
+    <s v="Novawerk GmbH"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="972085"/>
+    <n v="64.3"/>
+    <n v="4586"/>
+    <s v="SK14"/>
+    <n v="3.3273692943836743E-3"/>
+    <n v="0.93712979557311349"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0033"/>
+    <s v="Primaplast S.r.l."/>
+    <s v="IT"/>
+    <s v="Valves"/>
+    <s v="Quality risk"/>
+    <n v="962516"/>
+    <n v="100"/>
+    <n v="1082"/>
+    <s v="NT60"/>
+    <n v="3.2946153718584246E-3"/>
+    <n v="0.94042441094497187"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0062"/>
+    <s v="Rheinplast S.r.l."/>
+    <s v="IT"/>
+    <s v="Valves"/>
+    <s v="Reliable, lower spend"/>
+    <n v="948328"/>
+    <n v="100"/>
+    <n v="57"/>
+    <s v="missing"/>
+    <n v="3.2460509813486281E-3"/>
+    <n v="0.94367046192632054"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0008"/>
+    <s v="Polarparts GmbH"/>
+    <s v="DE"/>
+    <s v="Valves"/>
+    <s v="Delivery risk"/>
+    <n v="872158"/>
+    <n v="33.299999999999997"/>
+    <n v="211"/>
+    <s v="NT30"/>
+    <n v="2.9853271566283573E-3"/>
+    <n v="0.9466557890829489"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0047"/>
+    <s v="Lumenparts GmbH"/>
+    <s v="DE"/>
+    <s v="Electronic sensors"/>
+    <s v="Reliable, lower spend"/>
+    <n v="849030"/>
+    <n v="100"/>
+    <n v="167"/>
+    <s v="SK14"/>
+    <n v="2.9061618603420185E-3"/>
+    <n v="0.94956195094329088"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <s v="G0057"/>
+    <s v="Ventotronic GmbH"/>
+    <s v="AT"/>
+    <s v="Packaging"/>
+    <s v="Reliable, lower spend"/>
+    <n v="847714"/>
+    <n v="100"/>
+    <n v="83"/>
+    <s v="SK14"/>
+    <n v="2.9016572974782679E-3"/>
+    <n v="0.95246360824076914"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0111"/>
+    <s v="Teraplast GmbH"/>
+    <s v="DE"/>
+    <s v="Valves"/>
+    <s v="Delivery risk"/>
+    <n v="847410"/>
+    <n v="16.7"/>
+    <n v="73"/>
+    <s v="SK14"/>
+    <n v="2.9006167297650613E-3"/>
+    <n v="0.95536422497053419"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0099"/>
+    <s v="Boraflex  s.r.o."/>
+    <s v="CZ"/>
+    <s v="Rubber seals"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="840934"/>
+    <n v="50"/>
+    <n v="1333"/>
+    <s v="NT45"/>
+    <n v="2.8784498991376688E-3"/>
+    <n v="0.95824267486967185"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0115"/>
+    <s v="Deltatc s.r.o."/>
+    <s v="CZ"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Quality risk"/>
+    <n v="832309"/>
+    <n v="100"/>
+    <n v="4103"/>
+    <s v="NT30"/>
+    <n v="2.8489272131955348E-3"/>
+    <n v="0.96109160208286737"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0053"/>
+    <s v="Lumenform GmbH"/>
+    <s v="DE"/>
+    <s v="Plastic housings"/>
+    <s v="Delivery risk"/>
+    <n v="779982"/>
+    <n v="83.3"/>
+    <n v="303"/>
+    <s v="NT45"/>
+    <n v="2.6698160726397044E-3"/>
+    <n v="0.96376141815550709"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0071"/>
+    <s v="Ventometal GmbH"/>
+    <s v="AT"/>
+    <s v="Rubber seals"/>
+    <s v="Reliable, lower spend"/>
+    <n v="706783"/>
+    <n v="100"/>
+    <n v="110"/>
+    <s v="NT30"/>
+    <n v="2.4192617435639645E-3"/>
+    <n v="0.96618067989907108"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0045"/>
+    <s v="Novaform GmbH"/>
+    <s v="DE"/>
+    <s v="Plastic housings"/>
+    <s v="Quality risk"/>
+    <n v="691913"/>
+    <n v="90.9"/>
+    <n v="1193"/>
+    <s v="NT45"/>
+    <n v="2.3683629215396711E-3"/>
+    <n v="0.96854904282061072"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0100"/>
+    <s v="Aquaparts  GmbH"/>
+    <s v="AT"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="659886"/>
+    <n v="75"/>
+    <n v="1143"/>
+    <s v="NT45"/>
+    <n v="2.2587370592012687E-3"/>
+    <n v="0.97080777987981204"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0046"/>
+    <s v="Nordline GmbH"/>
+    <s v="DE"/>
+    <s v="Electronic sensors"/>
+    <s v="Quality risk"/>
+    <n v="652473"/>
+    <n v="87.5"/>
+    <n v="616"/>
+    <s v="NT60"/>
+    <n v="2.2333629524315252E-3"/>
+    <n v="0.97304114283224352"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0106"/>
+    <s v="Veltec GmbH"/>
+    <s v="AT"/>
+    <s v="Plastic housings"/>
+    <s v="Reliable, lower spend"/>
+    <n v="651488"/>
+    <n v="88.9"/>
+    <n v="213"/>
+    <s v="NT30"/>
+    <n v="2.2299913761239308E-3"/>
+    <n v="0.97527113420836742"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0025"/>
+    <s v="Cerroline GmbH"/>
+    <s v="DE"/>
+    <s v="Plastic housings"/>
+    <s v="Delivery risk"/>
+    <n v="649690"/>
+    <n v="83.3"/>
+    <n v="133"/>
+    <s v="SK14"/>
+    <n v="2.2238369657675301E-3"/>
+    <n v="0.97749497117413497"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0119"/>
+    <s v="Voltasal Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Electronic sensors"/>
+    <s v="Reliable, lower spend"/>
+    <n v="630560"/>
+    <n v="100"/>
+    <n v="70"/>
+    <s v="NT30"/>
+    <n v="2.1583565040779046E-3"/>
+    <n v="0.97965332767821289"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0095"/>
+    <s v="Cerrotec GmbH"/>
+    <s v="DE"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="623639"/>
+    <n v="66.7"/>
+    <n v="602"/>
+    <s v="NT60"/>
+    <n v="2.1346664740019036E-3"/>
+    <n v="0.98178799415221485"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0018"/>
+    <s v="Voltaflex GmbH"/>
+    <s v="DE"/>
+    <s v="Packaging"/>
+    <s v="Delivery risk"/>
+    <n v="543136"/>
+    <n v="80"/>
+    <n v="0"/>
+    <s v="NT45"/>
+    <n v="1.8591111364483265E-3"/>
+    <n v="0.98364710528866317"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0064"/>
+    <s v="Deltacast GmbH"/>
+    <s v="DE"/>
+    <s v="Valves"/>
+    <s v="Delivery risk"/>
+    <n v="535293"/>
+    <n v="71.400000000000006"/>
+    <n v="93"/>
+    <s v="NT30"/>
+    <n v="1.8322651740316127E-3"/>
+    <n v="0.98547937046269474"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0104"/>
+    <s v="VELAFORM GMBH"/>
+    <s v="DE"/>
+    <s v="Rubber seals"/>
+    <s v="Quality risk"/>
+    <n v="507867"/>
+    <n v="90.9"/>
+    <n v="5338"/>
+    <s v="NT30"/>
+    <n v="1.7383881671157908E-3"/>
+    <n v="0.98721775862981054"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0105"/>
+    <s v="Silbercast  GmbH"/>
+    <s v="DE"/>
+    <s v="Valves"/>
+    <s v="Reliable, lower spend"/>
+    <n v="426144"/>
+    <n v="100"/>
+    <n v="0"/>
+    <s v="NT45"/>
+    <n v="1.4586568670289497E-3"/>
+    <n v="0.98867641549683949"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0005"/>
+    <s v="Lumenflex SAS"/>
+    <s v="FR"/>
+    <s v="Valves"/>
+    <s v="Delivery risk"/>
+    <n v="420399"/>
+    <n v="83.3"/>
+    <n v="68"/>
+    <s v="SK14"/>
+    <n v="1.4389921910014066E-3"/>
+    <n v="0.9901154076878409"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0040"/>
+    <s v="Nordguss SAS"/>
+    <s v="FR"/>
+    <s v="Electronic sensors"/>
+    <s v="Reliable, lower spend"/>
+    <n v="415296"/>
+    <n v="100"/>
+    <n v="217"/>
+    <s v="NT45"/>
+    <n v="1.421525029683991E-3"/>
+    <n v="0.99153693271752485"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0096"/>
+    <s v="Boraetal Sp. z o.o."/>
+    <s v="PL"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Reliable, lower spend"/>
+    <n v="408703"/>
+    <n v="100"/>
+    <n v="0"/>
+    <s v="SK14"/>
+    <n v="1.3989577174038186E-3"/>
+    <n v="0.99293589043492869"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0055"/>
+    <s v="Atlasform s.r.o."/>
+    <s v="CZ"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Delivery risk"/>
+    <n v="402479"/>
+    <n v="75"/>
+    <n v="0"/>
+    <s v="NT60"/>
+    <n v="1.3776534626439528E-3"/>
+    <n v="0.99431354389757265"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0007"/>
+    <s v="Orbiscast s.r.o."/>
+    <s v="CZ"/>
+    <s v="Rubber seals"/>
+    <s v="Critical: quality and delivery"/>
+    <n v="390726"/>
+    <n v="66.7"/>
+    <n v="725"/>
+    <s v="NT60"/>
+    <n v="1.3374238826001385E-3"/>
+    <n v="0.99565096778017281"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0108"/>
+    <s v="Rheinmeal s.r.o."/>
+    <s v="CZ"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Reliable, lower spend"/>
+    <n v="387605"/>
+    <n v="87.5"/>
+    <n v="0"/>
+    <s v="NT30"/>
+    <n v="1.3267409489392224E-3"/>
+    <n v="0.99697770872911207"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0112"/>
+    <s v="Boracast GmbH"/>
+    <s v="DE"/>
+    <s v="Hoses &amp; connectors"/>
+    <s v="Reliable, lower spend"/>
+    <n v="322426"/>
+    <n v="100"/>
+    <n v="128"/>
+    <s v="SK14"/>
+    <n v="1.1036384391395306E-3"/>
+    <n v="0.99808134716825159"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0054"/>
+    <s v="Terratronic GmbH"/>
+    <s v="AT"/>
+    <s v="Brazed heat exchangers"/>
+    <s v="Delivery risk"/>
+    <n v="288832"/>
+    <n v="37.5"/>
+    <n v="500"/>
+    <s v="NT45"/>
+    <n v="9.8864886098996027E-4"/>
+    <n v="0.99906999602924151"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <s v="G0075"/>
+    <s v="Silberguss GmbH"/>
+    <s v="DE"/>
+    <s v="Valves"/>
+    <s v="Reliable, lower spend"/>
+    <n v="271699"/>
+    <n v="100"/>
+    <n v="192"/>
+    <s v="NT30"/>
+    <n v="9.3000397075847273E-4"/>
+    <n v="1"/>
+    <s v="C"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{17D90305-32B3-764B-9989-EC94EC235F08}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="D1:F18" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6345,18 +8233,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD49C0F8-9F96-4F47-B62A-6FDD67704BE5}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>297</v>
       </c>
       <c r="B1" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D1" s="8"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>299</v>
       </c>
@@ -6364,8 +8255,11 @@
         <f>COUNTIF(Suppliers!L:L,A2)</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D2" s="11"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="13"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>300</v>
       </c>
@@ -6373,8 +8267,11 @@
         <f>COUNTIF(Suppliers!L:L,A3)</f>
         <v>34</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D3" s="11"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="13"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>301</v>
       </c>
@@ -6382,8 +8279,11 @@
         <f>COUNTIF(Suppliers!L:L,A4)</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D4" s="11"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="13"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>302</v>
       </c>
@@ -6391,6 +8291,74 @@
         <f>SUM(B2:B4)</f>
         <v>120</v>
       </c>
+      <c r="D5" s="11"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="13"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D6" s="11"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="13"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D7" s="11"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="13"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D8" s="11"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="13"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D9" s="11"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="13"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D10" s="11"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="13"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D11" s="11"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="13"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D12" s="11"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="13"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="13"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D14" s="11"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="13"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D15" s="11"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D16" s="11"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="13"/>
+    </row>
+    <row r="17" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D17" s="11"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="13"/>
+    </row>
+    <row r="18" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D18" s="14"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
M6 step 3b: PivotTable spend by supplier segment with share of total (64% of spend at suppliers that miss a KPI target)
</commit_message>
<xml_diff>
--- a/excel/Spend_Analysis.xlsx
+++ b/excel/Spend_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F721CC40-A1A4-8F42-88B2-EF619393B6DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A78238C-2ABE-0C42-AE48-5021B71FFC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suppliers" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId5"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="307">
   <si>
     <t>Golden ID</t>
   </si>
@@ -948,6 +948,18 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of Spend (EUR)</t>
+  </si>
+  <si>
+    <t>Sum of Spend (EUR)2</t>
   </si>
 </sst>
 </file>
@@ -1000,7 +1012,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1008,123 +1020,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1135,15 +1036,11 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1188,7 +1085,13 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="Segment (M2)" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="5">
+        <s v="Strategic and reliable"/>
+        <s v="Quality risk"/>
+        <s v="Critical: quality and delivery"/>
+        <s v="Delivery risk"/>
+        <s v="Reliable, lower spend"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Spend (EUR)" numFmtId="3">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="271699" maxValue="8729465"/>
@@ -1227,7 +1130,7 @@
     <s v="KAPPATEC GMBH"/>
     <s v="AT"/>
     <s v="Plastic housings"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="8729465"/>
     <n v="87"/>
     <n v="117"/>
@@ -1241,7 +1144,7 @@
     <s v="Lumencast GmbH"/>
     <s v="AT"/>
     <s v="Packaging"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="8166335"/>
     <n v="94.9"/>
     <n v="699"/>
@@ -1255,7 +1158,7 @@
     <s v="Deltaarts SAS"/>
     <s v="FR"/>
     <s v="Valves"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="7892755"/>
     <n v="93.3"/>
     <n v="134"/>
@@ -1269,7 +1172,7 @@
     <s v="Krafttec GmbH"/>
     <s v="DE"/>
     <s v="Plastic housings"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="7297508"/>
     <n v="85.1"/>
     <n v="789"/>
@@ -1283,7 +1186,7 @@
     <s v="Velawerk s.r.o."/>
     <s v="CZ"/>
     <s v="Plastic housings"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="7016505"/>
     <n v="96.3"/>
     <n v="102"/>
@@ -1297,7 +1200,7 @@
     <s v="Kappawerk GmbH"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="6591040"/>
     <n v="92.4"/>
     <n v="117"/>
@@ -1311,7 +1214,7 @@
     <s v="TAUROGUSS GMBH"/>
     <s v="DE"/>
     <s v="Rubber seals"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="6508860"/>
     <n v="88.2"/>
     <n v="60"/>
@@ -1325,7 +1228,7 @@
     <s v="Ventoplast GmbH"/>
     <s v="DE"/>
     <s v="Electronic sensors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="6491982"/>
     <n v="58.8"/>
     <n v="911"/>
@@ -1339,7 +1242,7 @@
     <s v="Polarcast Sp. z o.o."/>
     <s v="PL"/>
     <s v="Valves"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="6425100"/>
     <n v="79.3"/>
     <n v="5265"/>
@@ -1353,7 +1256,7 @@
     <s v="Cerroparts"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="6072516"/>
     <n v="96.5"/>
     <n v="104"/>
@@ -1367,7 +1270,7 @@
     <s v="Orbisparts GmbH"/>
     <s v="DE"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="5969282"/>
     <n v="64.099999999999994"/>
     <n v="916"/>
@@ -1381,7 +1284,7 @@
     <s v="Deltaflex  Sp.  z  o.o."/>
     <s v="PL"/>
     <s v="Aluminium castings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="5915328"/>
     <n v="51.6"/>
     <n v="114"/>
@@ -1395,7 +1298,7 @@
     <s v="Polarplast  S.r.l."/>
     <s v="IT"/>
     <s v="Valves"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="5803633"/>
     <n v="88.9"/>
     <n v="50"/>
@@ -1409,7 +1312,7 @@
     <s v="Alpenguss SAS"/>
     <s v="FR"/>
     <s v="Fasteners"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="5528859"/>
     <n v="90.4"/>
     <n v="806"/>
@@ -1423,7 +1326,7 @@
     <s v="Orbisflex GmbH"/>
     <s v="DE"/>
     <s v="Plastic housings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="4891366"/>
     <n v="83.1"/>
     <n v="140"/>
@@ -1437,7 +1340,7 @@
     <s v="Terraparts GmbH"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="4886318"/>
     <n v="67.900000000000006"/>
     <n v="173"/>
@@ -1451,7 +1354,7 @@
     <s v="Velacast GmbH"/>
     <s v="AT"/>
     <s v="Plastic housings"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="4635149"/>
     <n v="91.8"/>
     <n v="24"/>
@@ -1465,7 +1368,7 @@
     <s v="Alpentronic GmbH"/>
     <s v="DE"/>
     <s v="Rubber seals"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="4527145"/>
     <n v="96.6"/>
     <n v="75"/>
@@ -1479,7 +1382,7 @@
     <s v="Ferrocast GmbH"/>
     <s v="DE"/>
     <s v="Aluminium castings"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="4516419"/>
     <n v="94.1"/>
     <n v="747"/>
@@ -1493,7 +1396,7 @@
     <s v="Boraline GmbH"/>
     <s v="DE"/>
     <s v="Fasteners"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="4112508"/>
     <n v="41.7"/>
     <n v="980"/>
@@ -1507,7 +1410,7 @@
     <s v="Velaline S.r.l."/>
     <s v="IT"/>
     <s v="Aluminium castings"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="4009816"/>
     <n v="73.8"/>
     <n v="893"/>
@@ -1521,7 +1424,7 @@
     <s v="Ferrotronic S.r.l."/>
     <s v="IT"/>
     <s v="Plastic housings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="3901204"/>
     <n v="70"/>
     <n v="146"/>
@@ -1535,7 +1438,7 @@
     <s v="Ferroform s.r.o."/>
     <s v="CZ"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="3850896"/>
     <n v="77.099999999999994"/>
     <n v="902"/>
@@ -1549,7 +1452,7 @@
     <s v="RHEINGUSS SAS"/>
     <s v="FR"/>
     <s v="Plastic housings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="3790329"/>
     <n v="58.8"/>
     <n v="164"/>
@@ -1563,7 +1466,7 @@
     <s v="Cerroform  S.r.l."/>
     <s v="IT"/>
     <s v="Valves"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="3669523"/>
     <n v="95.9"/>
     <n v="90"/>
@@ -1577,7 +1480,7 @@
     <s v="Primaparts GmbH"/>
     <s v="DE"/>
     <s v="Electronic sensors"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="3559963"/>
     <n v="90"/>
     <n v="87"/>
@@ -1591,7 +1494,7 @@
     <s v="NORDCAST SP. Z O.O."/>
     <s v="PL"/>
     <s v="Plastic housings"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="3489820"/>
     <n v="82.1"/>
     <n v="743"/>
@@ -1605,7 +1508,7 @@
     <s v="Voltacast GmbH"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="3460790"/>
     <n v="94.9"/>
     <n v="797"/>
@@ -1619,7 +1522,7 @@
     <s v="Voltatec GmbH"/>
     <s v="DE"/>
     <s v="Aluminium castings"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="3429954"/>
     <n v="86.5"/>
     <n v="5270"/>
@@ -1633,7 +1536,7 @@
     <s v="Voltawerk GmbH"/>
     <s v="DE"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="3295628"/>
     <n v="65.5"/>
     <n v="943"/>
@@ -1647,7 +1550,7 @@
     <s v="Ferroflex GmbH"/>
     <s v="DE"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="3104710"/>
     <n v="72.5"/>
     <n v="748"/>
@@ -1661,7 +1564,7 @@
     <s v="Terraseal  SAS"/>
     <s v="FR"/>
     <s v="Rubber seals"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="3090622"/>
     <n v="94.1"/>
     <n v="133"/>
@@ -1675,7 +1578,7 @@
     <s v="Novaseal GmbH"/>
     <s v="DE"/>
     <s v="Rubber seals"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="3030493"/>
     <n v="91.9"/>
     <n v="835"/>
@@ -1689,7 +1592,7 @@
     <s v="Silberline S.r.l."/>
     <s v="IT"/>
     <s v="Packaging"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="2959201"/>
     <n v="54.3"/>
     <n v="670"/>
@@ -1703,7 +1606,7 @@
     <s v="Aquametal GmbH"/>
     <s v="DE"/>
     <s v="Valves"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="2943032"/>
     <n v="75"/>
     <n v="85"/>
@@ -1717,7 +1620,7 @@
     <s v="Nordplast  s.r.o."/>
     <s v="CZ"/>
     <s v="Rubber seals"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="2923417"/>
     <n v="42.5"/>
     <n v="127"/>
@@ -1731,7 +1634,7 @@
     <s v="Ventoline S.r.l."/>
     <s v="IT"/>
     <s v="Electronic sensors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="2882552"/>
     <n v="81.8"/>
     <n v="869"/>
@@ -1745,7 +1648,7 @@
     <s v="Taurometal Sp. z o.o."/>
     <s v="PL"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="2871672"/>
     <n v="76.5"/>
     <n v="4588"/>
@@ -1759,7 +1662,7 @@
     <s v="Alpencast Sp. z o.o."/>
     <s v="PL"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="2865400"/>
     <n v="64.5"/>
     <n v="19"/>
@@ -1773,7 +1676,7 @@
     <s v="Kappaplast GmbH"/>
     <s v="DE"/>
     <s v="Fasteners"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="2825038"/>
     <n v="73.099999999999994"/>
     <n v="816"/>
@@ -1787,7 +1690,7 @@
     <s v="Atlasflex GmbH"/>
     <s v="AT"/>
     <s v="Electronic sensors"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2697901"/>
     <n v="96.9"/>
     <n v="113"/>
@@ -1801,7 +1704,7 @@
     <s v="Kraftflex s.r.o."/>
     <s v="CZ"/>
     <s v="Plastic housings"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="2629295"/>
     <n v="36.4"/>
     <n v="863"/>
@@ -1815,7 +1718,7 @@
     <s v="Silbermetal s.r.o."/>
     <s v="CZ"/>
     <s v="Valves"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2483150"/>
     <n v="90.9"/>
     <n v="68"/>
@@ -1829,7 +1732,7 @@
     <s v="Deltaguss GmbH"/>
     <s v="DE"/>
     <s v="Fasteners"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="2466796"/>
     <n v="51.6"/>
     <n v="68"/>
@@ -1843,7 +1746,7 @@
     <s v="Alpenwerk GmbH"/>
     <s v="AT"/>
     <s v="Electronic sensors"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="2435186"/>
     <n v="96"/>
     <n v="4612"/>
@@ -1857,7 +1760,7 @@
     <s v="FERROMETAL GMBH"/>
     <s v="DE"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2325849"/>
     <n v="90"/>
     <n v="189"/>
@@ -1871,7 +1774,7 @@
     <s v="Ferroparts GmbH"/>
     <s v="DE"/>
     <s v="Electronic sensors"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2314507"/>
     <n v="93.9"/>
     <n v="110"/>
@@ -1885,7 +1788,7 @@
     <s v="Voltaplast GmbH"/>
     <s v="DE"/>
     <s v="Fasteners"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="2304631"/>
     <n v="71.400000000000006"/>
     <n v="100"/>
@@ -1899,7 +1802,7 @@
     <s v="Kraftseal S.r.l."/>
     <s v="IT"/>
     <s v="Valves"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2255266"/>
     <n v="85.7"/>
     <n v="134"/>
@@ -1913,7 +1816,7 @@
     <s v="Velaguss Sp. z o.o."/>
     <s v="PL"/>
     <s v="Plastic housings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="2235309"/>
     <n v="65"/>
     <n v="76"/>
@@ -1927,7 +1830,7 @@
     <s v="Atlasplast Sp. z o.o."/>
     <s v="PL"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2128201"/>
     <n v="100"/>
     <n v="109"/>
@@ -1941,7 +1844,7 @@
     <s v="PRIMAFORM S.R.L."/>
     <s v="IT"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2119288"/>
     <n v="91.7"/>
     <n v="147"/>
@@ -1955,7 +1858,7 @@
     <s v="Vltatronic Sp. z o.o."/>
     <s v="PL"/>
     <s v="Valves"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="2096576"/>
     <n v="72.2"/>
     <n v="1167"/>
@@ -1969,7 +1872,7 @@
     <s v="Kraftcast  Sp.  z  o.o."/>
     <s v="PL"/>
     <s v="Electronic sensors"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2078432"/>
     <n v="94.6"/>
     <n v="167"/>
@@ -1983,7 +1886,7 @@
     <s v="Taurotec  GmbH"/>
     <s v="DE"/>
     <s v="Aluminium castings"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="2056747"/>
     <n v="94.7"/>
     <n v="107"/>
@@ -1997,7 +1900,7 @@
     <s v="Nordwerk GmbH"/>
     <s v="AT"/>
     <s v="Rubber seals"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="2053464"/>
     <n v="87.5"/>
     <n v="1013"/>
@@ -2011,7 +1914,7 @@
     <s v="KRAFTFORM SAS"/>
     <s v="FR"/>
     <s v="Rubber seals"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="1985456"/>
     <n v="86.7"/>
     <n v="730"/>
@@ -2025,7 +1928,7 @@
     <s v="Ventoseal GmbH"/>
     <s v="DE"/>
     <s v="Valves"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1970618"/>
     <n v="73.7"/>
     <n v="718"/>
@@ -2039,7 +1942,7 @@
     <s v="Tauroparts S.r.l."/>
     <s v="IT"/>
     <s v="Electronic sensors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1919165"/>
     <n v="72.2"/>
     <n v="810"/>
@@ -2053,7 +1956,7 @@
     <s v="Boratronic SAS"/>
     <s v="FR"/>
     <s v="Electronic sensors"/>
-    <s v="Strategic and reliable"/>
+    <x v="0"/>
     <n v="1917140"/>
     <n v="88"/>
     <n v="109"/>
@@ -2067,7 +1970,7 @@
     <s v="Deltametal Sp. z o.o."/>
     <s v="PL"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1878888"/>
     <n v="68.8"/>
     <n v="145"/>
@@ -2081,7 +1984,7 @@
     <s v="Novametal Sp. z o.o."/>
     <s v="PL"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="1870250"/>
     <n v="100"/>
     <n v="0"/>
@@ -2095,7 +1998,7 @@
     <s v="Kraftguss s.r.o."/>
     <s v="CZ"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1863627"/>
     <n v="57.1"/>
     <n v="4508"/>
@@ -2109,7 +2012,7 @@
     <s v="Velaseal s.r.o."/>
     <s v="CZ"/>
     <s v="Valves"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1818970"/>
     <n v="44.4"/>
     <n v="4723"/>
@@ -2123,7 +2026,7 @@
     <s v="RHEINSEAL GMBH"/>
     <s v="DE"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1780307"/>
     <n v="79.3"/>
     <n v="135"/>
@@ -2137,7 +2040,7 @@
     <s v="Nordtronic"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1727420"/>
     <n v="42.9"/>
     <n v="165"/>
@@ -2151,7 +2054,7 @@
     <s v="Atlasparts Sp. z o.o."/>
     <s v="PL"/>
     <s v="Electronic sensors"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="1719814"/>
     <n v="94.1"/>
     <n v="110"/>
@@ -2165,7 +2068,7 @@
     <s v="Boratc S.r.l."/>
     <s v="IT"/>
     <s v="Electronic sensors"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="1693890"/>
     <n v="94.7"/>
     <n v="705"/>
@@ -2179,7 +2082,7 @@
     <s v="Orbisguss"/>
     <s v="DE"/>
     <s v="Rubber seals"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1625687"/>
     <n v="70.599999999999994"/>
     <n v="211"/>
@@ -2193,7 +2096,7 @@
     <s v="Tauroseal"/>
     <s v="DE"/>
     <s v="Aluminium castings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1545398"/>
     <n v="54.2"/>
     <n v="0"/>
@@ -2207,7 +2110,7 @@
     <s v="Boraseal GmbH"/>
     <s v="DE"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1544505"/>
     <n v="63.6"/>
     <n v="861"/>
@@ -2221,7 +2124,7 @@
     <s v="Atlasguss  GmbH"/>
     <s v="DE"/>
     <s v="Rubber seals"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="1532145"/>
     <n v="87.5"/>
     <n v="118"/>
@@ -2235,7 +2138,7 @@
     <s v="Silberwerk s.r.o."/>
     <s v="CZ"/>
     <s v="Electronic sensors"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1479272"/>
     <n v="63.6"/>
     <n v="53"/>
@@ -2249,7 +2152,7 @@
     <s v="Cerrocast s.r.o."/>
     <s v="CZ"/>
     <s v="Valves"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1406564"/>
     <n v="52.2"/>
     <n v="885"/>
@@ -2263,7 +2166,7 @@
     <s v="Deltaform Sp. z o.o."/>
     <s v="PL"/>
     <s v="Packaging"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="1405509"/>
     <n v="95.2"/>
     <n v="5227"/>
@@ -2277,7 +2180,7 @@
     <s v="Cerrowerk Sp. z o.o."/>
     <s v="PL"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1292882"/>
     <n v="57.1"/>
     <n v="248"/>
@@ -2291,7 +2194,7 @@
     <s v="Deltaplast GmbH"/>
     <s v="DE"/>
     <s v="Aluminium castings"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="1268156"/>
     <n v="100"/>
     <n v="81"/>
@@ -2305,7 +2208,7 @@
     <s v="Aquaplast s.r.o."/>
     <s v="CZ"/>
     <s v="Rubber seals"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="1172222"/>
     <n v="85.7"/>
     <n v="75"/>
@@ -2319,7 +2222,7 @@
     <s v="Ventoguss GmbH"/>
     <s v="DE"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1150286"/>
     <n v="58.3"/>
     <n v="1048"/>
@@ -2333,7 +2236,7 @@
     <s v="Tauroform Sp. z o.o."/>
     <s v="PL"/>
     <s v="Rubber seals"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1138729"/>
     <n v="46.2"/>
     <n v="550"/>
@@ -2347,7 +2250,7 @@
     <s v="Atlastronc GmbH"/>
     <s v="DE"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="1113399"/>
     <n v="100"/>
     <n v="288"/>
@@ -2361,7 +2264,7 @@
     <s v="Kappaform GmbH"/>
     <s v="AT"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1111745"/>
     <n v="80"/>
     <n v="74"/>
@@ -2375,7 +2278,7 @@
     <s v="Orbistronic"/>
     <s v="IT"/>
     <s v="Electronic sensors"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1093804"/>
     <n v="69.2"/>
     <n v="81"/>
@@ -2389,7 +2292,7 @@
     <s v="Velaparts s.r.o."/>
     <s v="CZ"/>
     <s v="Rubber seals"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="1061536"/>
     <n v="90.9"/>
     <n v="503"/>
@@ -2403,7 +2306,7 @@
     <s v="Novaline GmbH"/>
     <s v="DE"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="1055719"/>
     <n v="76.900000000000006"/>
     <n v="725"/>
@@ -2417,7 +2320,7 @@
     <s v="Aquatronic GmbH"/>
     <s v="DE"/>
     <s v="Rubber seals"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1037511"/>
     <n v="70"/>
     <n v="116"/>
@@ -2431,7 +2334,7 @@
     <s v="Atlaswerk GmbH"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="1011810"/>
     <n v="80"/>
     <n v="0"/>
@@ -2445,7 +2348,7 @@
     <s v="Polarmetal s.r.o."/>
     <s v="CZ"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="1005997"/>
     <n v="100"/>
     <n v="5294"/>
@@ -2459,7 +2362,7 @@
     <s v="Lumenwerk s.r.o."/>
     <s v="CZ"/>
     <s v="Plastic housings"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="997560"/>
     <n v="72.7"/>
     <n v="1095"/>
@@ -2473,7 +2376,7 @@
     <s v="Novawerk GmbH"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="972085"/>
     <n v="64.3"/>
     <n v="4586"/>
@@ -2487,7 +2390,7 @@
     <s v="Primaplast S.r.l."/>
     <s v="IT"/>
     <s v="Valves"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="962516"/>
     <n v="100"/>
     <n v="1082"/>
@@ -2501,7 +2404,7 @@
     <s v="Rheinplast S.r.l."/>
     <s v="IT"/>
     <s v="Valves"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="948328"/>
     <n v="100"/>
     <n v="57"/>
@@ -2515,7 +2418,7 @@
     <s v="Polarparts GmbH"/>
     <s v="DE"/>
     <s v="Valves"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="872158"/>
     <n v="33.299999999999997"/>
     <n v="211"/>
@@ -2529,7 +2432,7 @@
     <s v="Lumenparts GmbH"/>
     <s v="DE"/>
     <s v="Electronic sensors"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="849030"/>
     <n v="100"/>
     <n v="167"/>
@@ -2543,7 +2446,7 @@
     <s v="Ventotronic GmbH"/>
     <s v="AT"/>
     <s v="Packaging"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="847714"/>
     <n v="100"/>
     <n v="83"/>
@@ -2557,7 +2460,7 @@
     <s v="Teraplast GmbH"/>
     <s v="DE"/>
     <s v="Valves"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="847410"/>
     <n v="16.7"/>
     <n v="73"/>
@@ -2571,7 +2474,7 @@
     <s v="Boraflex  s.r.o."/>
     <s v="CZ"/>
     <s v="Rubber seals"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="840934"/>
     <n v="50"/>
     <n v="1333"/>
@@ -2585,7 +2488,7 @@
     <s v="Deltatc s.r.o."/>
     <s v="CZ"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="832309"/>
     <n v="100"/>
     <n v="4103"/>
@@ -2599,7 +2502,7 @@
     <s v="Lumenform GmbH"/>
     <s v="DE"/>
     <s v="Plastic housings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="779982"/>
     <n v="83.3"/>
     <n v="303"/>
@@ -2613,7 +2516,7 @@
     <s v="Ventometal GmbH"/>
     <s v="AT"/>
     <s v="Rubber seals"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="706783"/>
     <n v="100"/>
     <n v="110"/>
@@ -2627,7 +2530,7 @@
     <s v="Novaform GmbH"/>
     <s v="DE"/>
     <s v="Plastic housings"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="691913"/>
     <n v="90.9"/>
     <n v="1193"/>
@@ -2641,7 +2544,7 @@
     <s v="Aquaparts  GmbH"/>
     <s v="AT"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="659886"/>
     <n v="75"/>
     <n v="1143"/>
@@ -2655,7 +2558,7 @@
     <s v="Nordline GmbH"/>
     <s v="DE"/>
     <s v="Electronic sensors"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="652473"/>
     <n v="87.5"/>
     <n v="616"/>
@@ -2669,7 +2572,7 @@
     <s v="Veltec GmbH"/>
     <s v="AT"/>
     <s v="Plastic housings"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="651488"/>
     <n v="88.9"/>
     <n v="213"/>
@@ -2683,7 +2586,7 @@
     <s v="Cerroline GmbH"/>
     <s v="DE"/>
     <s v="Plastic housings"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="649690"/>
     <n v="83.3"/>
     <n v="133"/>
@@ -2697,7 +2600,7 @@
     <s v="Voltasal Sp. z o.o."/>
     <s v="PL"/>
     <s v="Electronic sensors"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="630560"/>
     <n v="100"/>
     <n v="70"/>
@@ -2711,7 +2614,7 @@
     <s v="Cerrotec GmbH"/>
     <s v="DE"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="623639"/>
     <n v="66.7"/>
     <n v="602"/>
@@ -2725,7 +2628,7 @@
     <s v="Voltaflex GmbH"/>
     <s v="DE"/>
     <s v="Packaging"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="543136"/>
     <n v="80"/>
     <n v="0"/>
@@ -2739,7 +2642,7 @@
     <s v="Deltacast GmbH"/>
     <s v="DE"/>
     <s v="Valves"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="535293"/>
     <n v="71.400000000000006"/>
     <n v="93"/>
@@ -2753,7 +2656,7 @@
     <s v="VELAFORM GMBH"/>
     <s v="DE"/>
     <s v="Rubber seals"/>
-    <s v="Quality risk"/>
+    <x v="1"/>
     <n v="507867"/>
     <n v="90.9"/>
     <n v="5338"/>
@@ -2767,7 +2670,7 @@
     <s v="Silbercast  GmbH"/>
     <s v="DE"/>
     <s v="Valves"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="426144"/>
     <n v="100"/>
     <n v="0"/>
@@ -2781,7 +2684,7 @@
     <s v="Lumenflex SAS"/>
     <s v="FR"/>
     <s v="Valves"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="420399"/>
     <n v="83.3"/>
     <n v="68"/>
@@ -2795,7 +2698,7 @@
     <s v="Nordguss SAS"/>
     <s v="FR"/>
     <s v="Electronic sensors"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="415296"/>
     <n v="100"/>
     <n v="217"/>
@@ -2809,7 +2712,7 @@
     <s v="Boraetal Sp. z o.o."/>
     <s v="PL"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="408703"/>
     <n v="100"/>
     <n v="0"/>
@@ -2823,7 +2726,7 @@
     <s v="Atlasform s.r.o."/>
     <s v="CZ"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="402479"/>
     <n v="75"/>
     <n v="0"/>
@@ -2837,7 +2740,7 @@
     <s v="Orbiscast s.r.o."/>
     <s v="CZ"/>
     <s v="Rubber seals"/>
-    <s v="Critical: quality and delivery"/>
+    <x v="2"/>
     <n v="390726"/>
     <n v="66.7"/>
     <n v="725"/>
@@ -2851,7 +2754,7 @@
     <s v="Rheinmeal s.r.o."/>
     <s v="CZ"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="387605"/>
     <n v="87.5"/>
     <n v="0"/>
@@ -2865,7 +2768,7 @@
     <s v="Boracast GmbH"/>
     <s v="DE"/>
     <s v="Hoses &amp; connectors"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="322426"/>
     <n v="100"/>
     <n v="128"/>
@@ -2879,7 +2782,7 @@
     <s v="Terratronic GmbH"/>
     <s v="AT"/>
     <s v="Brazed heat exchangers"/>
-    <s v="Delivery risk"/>
+    <x v="3"/>
     <n v="288832"/>
     <n v="37.5"/>
     <n v="500"/>
@@ -2893,7 +2796,7 @@
     <s v="Silberguss GmbH"/>
     <s v="DE"/>
     <s v="Valves"/>
-    <s v="Reliable, lower spend"/>
+    <x v="4"/>
     <n v="271699"/>
     <n v="100"/>
     <n v="192"/>
@@ -2906,15 +2809,24 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{17D90305-32B3-764B-9989-EC94EC235F08}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="D1:F18" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{17D90305-32B3-764B-9989-EC94EC235F08}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="D1:F7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="3" showAll="0"/>
     <pivotField numFmtId="164" showAll="0"/>
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
@@ -2922,6 +2834,44 @@
     <pivotField numFmtId="9" showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of Spend (EUR)" fld="5" baseField="0" baseItem="0" numFmtId="3"/>
+    <dataField name="Sum of Spend (EUR)2" fld="5" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
+  </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -7276,7 +7226,7 @@
         <v>0.95824267486967185</v>
       </c>
       <c r="L98" t="str">
-        <f t="shared" ref="L98:L129" si="7">IF(K98&lt;=80%,"A",IF(K98&lt;=95%,"B","C"))</f>
+        <f t="shared" ref="L98:L121" si="7">IF(K98&lt;=80%,"A",IF(K98&lt;=95%,"B","C"))</f>
         <v>C</v>
       </c>
     </row>
@@ -8233,8 +8183,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD49C0F8-9F96-4F47-B62A-6FDD67704BE5}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -8243,9 +8198,15 @@
       <c r="B1" t="s">
         <v>298</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="10"/>
+      <c r="D1" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="E1" t="s">
+        <v>305</v>
+      </c>
+      <c r="F1" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -8255,9 +8216,15 @@
         <f>COUNTIF(Suppliers!L:L,A2)</f>
         <v>60</v>
       </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="13"/>
+      <c r="D2" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2">
+        <v>75367089</v>
+      </c>
+      <c r="F2" s="10">
+        <v>0.25797552451244654</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -8267,9 +8234,15 @@
         <f>COUNTIF(Suppliers!L:L,A3)</f>
         <v>34</v>
       </c>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="13"/>
+      <c r="D3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="2">
+        <v>60047233</v>
+      </c>
+      <c r="F3" s="10">
+        <v>0.20553688133949408</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -8279,9 +8252,15 @@
         <f>COUNTIF(Suppliers!L:L,A4)</f>
         <v>26</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="13"/>
+      <c r="D4" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="2">
+        <v>50718474</v>
+      </c>
+      <c r="F4" s="10">
+        <v>0.17360528456420657</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -8291,74 +8270,37 @@
         <f>SUM(B2:B4)</f>
         <v>120</v>
       </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="13"/>
+      <c r="D5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="2">
+        <v>15541762</v>
+      </c>
+      <c r="F5" s="10">
+        <v>5.3198209682711904E-2</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="13"/>
+      <c r="D6" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="2">
+        <v>90473657</v>
+      </c>
+      <c r="F6" s="10">
+        <v>0.30968409990114093</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D7" s="11"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D8" s="11"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="13"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D9" s="11"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D10" s="11"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="13"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D11" s="11"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D12" s="11"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D13" s="11"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D14" s="11"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="13"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D15" s="11"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="13"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D16" s="11"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="13"/>
-    </row>
-    <row r="17" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D17" s="11"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="13"/>
-    </row>
-    <row r="18" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D18" s="14"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="16"/>
+      <c r="D7" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="E7" s="2">
+        <v>292148215</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
M6 step 3c (part 1): net payment days with XLOOKUP and cash effect of a 60-day standard term
</commit_message>
<xml_diff>
--- a/excel/Spend_Analysis.xlsx
+++ b/excel/Spend_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A78238C-2ABE-0C42-AE48-5021B71FFC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC0AB29-2118-CC40-8BC5-DBFA9AD6005B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suppliers" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="308">
   <si>
     <t>Golden ID</t>
   </si>
@@ -960,6 +960,9 @@
   </si>
   <si>
     <t>Sum of Spend (EUR)2</t>
+  </si>
+  <si>
+    <t>Cash effect (EUR)</t>
   </si>
 </sst>
 </file>
@@ -1046,7 +1049,13 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -2885,12 +2894,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSpend" displayName="tblSpend" ref="A1:L121">
-  <autoFilter ref="A1:L121" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSpend" displayName="tblSpend" ref="A1:N121">
+  <autoFilter ref="A1:N121" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I121">
     <sortCondition descending="1" ref="F1:F121"/>
   </sortState>
-  <tableColumns count="12">
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Golden ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Supplier"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Country"/>
@@ -2903,11 +2912,17 @@
     <tableColumn id="10" xr3:uid="{5D1E5103-053F-9149-A678-5C4D8626A5EA}" name="Spend share" dataCellStyle="Percent">
       <calculatedColumnFormula>F2/SUM($F$2:$F$121)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{B3C0593A-4800-A24E-858E-2C3789403277}" name="Cumulative share" dataDxfId="1">
+    <tableColumn id="11" xr3:uid="{B3C0593A-4800-A24E-858E-2C3789403277}" name="Cumulative share" dataDxfId="3">
       <calculatedColumnFormula>SUM($J$2:J2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{DFA46FC0-C59B-9B4C-8696-052595BBF44D}" name="ABC class" dataDxfId="0">
+    <tableColumn id="12" xr3:uid="{DFA46FC0-C59B-9B4C-8696-052595BBF44D}" name="ABC class" dataDxfId="2">
       <calculatedColumnFormula>IF(K2&lt;=80%,"A",IF(K2&lt;=95%,"B","C"))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{A6793419-9AA1-3242-B71C-8AD377F8F478}" name="Net days" dataDxfId="1">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(I2,Terms!A:A,Terms!C:C,"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="14" xr3:uid="{0BFB64A9-2F55-0641-BBF7-61A0DC5F3A72}" name="Cash effect (EUR)" dataDxfId="0">
+      <calculatedColumnFormula>IF(M2="",0,MAX(0,Settings!$B$5-M2)*F2/Settings!$B$4)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3199,7 +3214,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:N121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
@@ -3212,10 +3227,12 @@
     <col min="9" max="9" width="16.1640625" customWidth="1"/>
     <col min="10" max="10" width="15" style="7" customWidth="1"/>
     <col min="11" max="11" width="18.6640625" customWidth="1"/>
-    <col min="12" max="12" width="12.1640625" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" customWidth="1"/>
+    <col min="13" max="13" width="15.5" customWidth="1"/>
+    <col min="14" max="14" width="21.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3252,8 +3269,14 @@
       <c r="L1" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M1" t="s">
+        <v>276</v>
+      </c>
+      <c r="N1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>228</v>
       </c>
@@ -3293,8 +3316,16 @@
         <f t="shared" ref="L2:L33" si="1">IF(K2&lt;=80%,"A",IF(K2&lt;=95%,"B","C"))</f>
         <v>A</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M2">
+        <f>_xlfn.XLOOKUP(I2,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N2">
+        <f>IF(M2="",0,MAX(0,Settings!$B$5-M2)*F2/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>61</v>
       </c>
@@ -3334,8 +3365,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M3" t="str">
+        <f>_xlfn.XLOOKUP(I3,Terms!A:A,Terms!C:C,"")</f>
+        <v/>
+      </c>
+      <c r="N3">
+        <f>IF(M3="",0,MAX(0,Settings!$B$5-M3)*F3/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>236</v>
       </c>
@@ -3375,8 +3414,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M4">
+        <f>_xlfn.XLOOKUP(I4,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N4">
+        <f>IF(M4="",0,MAX(0,Settings!$B$5-M4)*F4/Settings!$B$4)</f>
+        <v>928559.4117647059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>136</v>
       </c>
@@ -3416,8 +3463,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M5">
+        <f>_xlfn.XLOOKUP(I5,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N5">
+        <f>IF(M5="",0,MAX(0,Settings!$B$5-M5)*F5/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -3457,8 +3512,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M6">
+        <f>_xlfn.XLOOKUP(I6,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N6">
+        <f>IF(M6="",0,MAX(0,Settings!$B$5-M6)*F6/Settings!$B$4)</f>
+        <v>412735.5882352941</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>198</v>
       </c>
@@ -3498,8 +3561,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M7">
+        <f>_xlfn.XLOOKUP(I7,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N7">
+        <f>IF(M7="",0,MAX(0,Settings!$B$5-M7)*F7/Settings!$B$4)</f>
+        <v>775416.4705882353</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>238</v>
       </c>
@@ -3539,8 +3610,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M8">
+        <f>_xlfn.XLOOKUP(I8,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N8">
+        <f>IF(M8="",0,MAX(0,Settings!$B$5-M8)*F8/Settings!$B$4)</f>
+        <v>765748.23529411759</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>120</v>
       </c>
@@ -3580,8 +3659,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M9">
+        <f>_xlfn.XLOOKUP(I9,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N9">
+        <f>IF(M9="",0,MAX(0,Settings!$B$5-M9)*F9/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>158</v>
       </c>
@@ -3621,8 +3708,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M10">
+        <f>_xlfn.XLOOKUP(I10,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N10">
+        <f>IF(M10="",0,MAX(0,Settings!$B$5-M10)*F10/Settings!$B$4)</f>
+        <v>377947.0588235294</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>220</v>
       </c>
@@ -3662,8 +3757,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M11">
+        <f>_xlfn.XLOOKUP(I11,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N11">
+        <f>IF(M11="",0,MAX(0,Settings!$B$5-M11)*F11/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -3703,8 +3806,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M12">
+        <f>_xlfn.XLOOKUP(I12,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N12">
+        <f>IF(M12="",0,MAX(0,Settings!$B$5-M12)*F12/Settings!$B$4)</f>
+        <v>351134.23529411765</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>266</v>
       </c>
@@ -3744,8 +3855,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M13">
+        <f>_xlfn.XLOOKUP(I13,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N13">
+        <f>IF(M13="",0,MAX(0,Settings!$B$5-M13)*F13/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>206</v>
       </c>
@@ -3785,8 +3904,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M14">
+        <f>_xlfn.XLOOKUP(I14,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N14">
+        <f>IF(M14="",0,MAX(0,Settings!$B$5-M14)*F14/Settings!$B$4)</f>
+        <v>682780.3529411765</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>180</v>
       </c>
@@ -3826,8 +3953,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M15">
+        <f>_xlfn.XLOOKUP(I15,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N15">
+        <f>IF(M15="",0,MAX(0,Settings!$B$5-M15)*F15/Settings!$B$4)</f>
+        <v>650454</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>260</v>
       </c>
@@ -3867,8 +4002,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M16">
+        <f>_xlfn.XLOOKUP(I16,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N16">
+        <f>IF(M16="",0,MAX(0,Settings!$B$5-M16)*F16/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>172</v>
       </c>
@@ -3908,8 +4051,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M17">
+        <f>_xlfn.XLOOKUP(I17,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N17">
+        <f>IF(M17="",0,MAX(0,Settings!$B$5-M17)*F17/Settings!$B$4)</f>
+        <v>574860.9411764706</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>76</v>
       </c>
@@ -3949,8 +4100,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M18">
+        <f>_xlfn.XLOOKUP(I18,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N18">
+        <f>IF(M18="",0,MAX(0,Settings!$B$5-M18)*F18/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -3990,8 +4149,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M19">
+        <f>_xlfn.XLOOKUP(I19,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N19">
+        <f>IF(M19="",0,MAX(0,Settings!$B$5-M19)*F19/Settings!$B$4)</f>
+        <v>266302.64705882355</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>128</v>
       </c>
@@ -4031,8 +4198,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M20">
+        <f>_xlfn.XLOOKUP(I20,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N20">
+        <f>IF(M20="",0,MAX(0,Settings!$B$5-M20)*F20/Settings!$B$4)</f>
+        <v>265671.70588235295</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>148</v>
       </c>
@@ -4072,8 +4247,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M21">
+        <f>_xlfn.XLOOKUP(I21,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N21">
+        <f>IF(M21="",0,MAX(0,Settings!$B$5-M21)*F21/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>192</v>
       </c>
@@ -4113,8 +4296,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M22">
+        <f>_xlfn.XLOOKUP(I22,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N22">
+        <f>IF(M22="",0,MAX(0,Settings!$B$5-M22)*F22/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>196</v>
       </c>
@@ -4154,8 +4345,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M23">
+        <f>_xlfn.XLOOKUP(I23,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N23">
+        <f>IF(M23="",0,MAX(0,Settings!$B$5-M23)*F23/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>15</v>
       </c>
@@ -4195,8 +4394,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M24">
+        <f>_xlfn.XLOOKUP(I24,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N24">
+        <f>IF(M24="",0,MAX(0,Settings!$B$5-M24)*F24/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>234</v>
       </c>
@@ -4236,8 +4443,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M25">
+        <f>_xlfn.XLOOKUP(I25,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N25">
+        <f>IF(M25="",0,MAX(0,Settings!$B$5-M25)*F25/Settings!$B$4)</f>
+        <v>445921.0588235294</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>268</v>
       </c>
@@ -4277,8 +4492,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M26">
+        <f>_xlfn.XLOOKUP(I26,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N26">
+        <f>IF(M26="",0,MAX(0,Settings!$B$5-M26)*F26/Settings!$B$4)</f>
+        <v>431708.5882352941</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>190</v>
       </c>
@@ -4318,8 +4541,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M27">
+        <f>_xlfn.XLOOKUP(I27,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N27">
+        <f>IF(M27="",0,MAX(0,Settings!$B$5-M27)*F27/Settings!$B$4)</f>
+        <v>418819.17647058825</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>80</v>
       </c>
@@ -4359,8 +4590,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M28">
+        <f>_xlfn.XLOOKUP(I28,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N28">
+        <f>IF(M28="",0,MAX(0,Settings!$B$5-M28)*F28/Settings!$B$4)</f>
+        <v>410567.0588235294</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>96</v>
       </c>
@@ -4400,8 +4639,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M29">
+        <f>_xlfn.XLOOKUP(I29,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N29">
+        <f>IF(M29="",0,MAX(0,Settings!$B$5-M29)*F29/Settings!$B$4)</f>
+        <v>203575.88235294117</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>202</v>
       </c>
@@ -4441,8 +4688,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M30">
+        <f>_xlfn.XLOOKUP(I30,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N30">
+        <f>IF(M30="",0,MAX(0,Settings!$B$5-M30)*F30/Settings!$B$4)</f>
+        <v>403524</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -4482,8 +4737,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M31">
+        <f>_xlfn.XLOOKUP(I31,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N31">
+        <f>IF(M31="",0,MAX(0,Settings!$B$5-M31)*F31/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>106</v>
       </c>
@@ -4523,8 +4786,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M32">
+        <f>_xlfn.XLOOKUP(I32,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N32">
+        <f>IF(M32="",0,MAX(0,Settings!$B$5-M32)*F32/Settings!$B$4)</f>
+        <v>365260</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>204</v>
       </c>
@@ -4564,8 +4835,16 @@
         <f t="shared" si="1"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M33">
+        <f>_xlfn.XLOOKUP(I33,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N33">
+        <f>IF(M33="",0,MAX(0,Settings!$B$5-M33)*F33/Settings!$B$4)</f>
+        <v>363602.5882352941</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>88</v>
       </c>
@@ -4605,8 +4884,16 @@
         <f t="shared" ref="L34:L65" si="3">IF(K34&lt;=80%,"A",IF(K34&lt;=95%,"B","C"))</f>
         <v>A</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M34">
+        <f>_xlfn.XLOOKUP(I34,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N34">
+        <f>IF(M34="",0,MAX(0,Settings!$B$5-M34)*F34/Settings!$B$4)</f>
+        <v>356528.5882352941</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>59</v>
       </c>
@@ -4646,8 +4933,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M35">
+        <f>_xlfn.XLOOKUP(I35,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N35">
+        <f>IF(M35="",0,MAX(0,Settings!$B$5-M35)*F35/Settings!$B$4)</f>
+        <v>348141.29411764705</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -4687,8 +4982,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M36">
+        <f>_xlfn.XLOOKUP(I36,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N36">
+        <f>IF(M36="",0,MAX(0,Settings!$B$5-M36)*F36/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>214</v>
       </c>
@@ -4728,8 +5031,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M37">
+        <f>_xlfn.XLOOKUP(I37,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N37">
+        <f>IF(M37="",0,MAX(0,Settings!$B$5-M37)*F37/Settings!$B$4)</f>
+        <v>343931.4117647059</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>26</v>
       </c>
@@ -4769,8 +5080,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M38">
+        <f>_xlfn.XLOOKUP(I38,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N38">
+        <f>IF(M38="",0,MAX(0,Settings!$B$5-M38)*F38/Settings!$B$4)</f>
+        <v>339123.76470588235</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -4810,8 +5129,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M39">
+        <f>_xlfn.XLOOKUP(I39,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N39">
+        <f>IF(M39="",0,MAX(0,Settings!$B$5-M39)*F39/Settings!$B$4)</f>
+        <v>337843.76470588235</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>150</v>
       </c>
@@ -4851,8 +5178,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M40">
+        <f>_xlfn.XLOOKUP(I40,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N40">
+        <f>IF(M40="",0,MAX(0,Settings!$B$5-M40)*F40/Settings!$B$4)</f>
+        <v>337105.8823529412</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -4892,8 +5227,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M41">
+        <f>_xlfn.XLOOKUP(I41,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N41">
+        <f>IF(M41="",0,MAX(0,Settings!$B$5-M41)*F41/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>132</v>
       </c>
@@ -4933,8 +5276,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M42">
+        <f>_xlfn.XLOOKUP(I42,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N42">
+        <f>IF(M42="",0,MAX(0,Settings!$B$5-M42)*F42/Settings!$B$4)</f>
+        <v>317400.1176470588</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>154</v>
       </c>
@@ -4974,8 +5325,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M43">
+        <f>_xlfn.XLOOKUP(I43,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N43">
+        <f>IF(M43="",0,MAX(0,Settings!$B$5-M43)*F43/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>92</v>
       </c>
@@ -5015,8 +5374,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M44">
+        <f>_xlfn.XLOOKUP(I44,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N44">
+        <f>IF(M44="",0,MAX(0,Settings!$B$5-M44)*F44/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -5056,8 +5423,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M45">
+        <f>_xlfn.XLOOKUP(I45,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N45">
+        <f>IF(M45="",0,MAX(0,Settings!$B$5-M45)*F45/Settings!$B$4)</f>
+        <v>145105.64705882352</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>102</v>
       </c>
@@ -5097,8 +5472,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M46">
+        <f>_xlfn.XLOOKUP(I46,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N46">
+        <f>IF(M46="",0,MAX(0,Settings!$B$5-M46)*F46/Settings!$B$4)</f>
+        <v>286492.4705882353</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>258</v>
       </c>
@@ -5138,8 +5521,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M47">
+        <f>_xlfn.XLOOKUP(I47,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N47">
+        <f>IF(M47="",0,MAX(0,Settings!$B$5-M47)*F47/Settings!$B$4)</f>
+        <v>136814.64705882352</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>110</v>
       </c>
@@ -5179,8 +5570,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M48">
+        <f>_xlfn.XLOOKUP(I48,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N48">
+        <f>IF(M48="",0,MAX(0,Settings!$B$5-M48)*F48/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>134</v>
       </c>
@@ -5220,8 +5619,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M49" t="str">
+        <f>_xlfn.XLOOKUP(I49,Terms!A:A,Terms!C:C,"")</f>
+        <v/>
+      </c>
+      <c r="N49">
+        <f>IF(M49="",0,MAX(0,Settings!$B$5-M49)*F49/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>94</v>
       </c>
@@ -5261,8 +5668,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M50">
+        <f>_xlfn.XLOOKUP(I50,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N50">
+        <f>IF(M50="",0,MAX(0,Settings!$B$5-M50)*F50/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>73</v>
       </c>
@@ -5302,8 +5717,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M51">
+        <f>_xlfn.XLOOKUP(I51,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N51">
+        <f>IF(M51="",0,MAX(0,Settings!$B$5-M51)*F51/Settings!$B$4)</f>
+        <v>131488.76470588235</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>114</v>
       </c>
@@ -5343,8 +5766,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M52">
+        <f>_xlfn.XLOOKUP(I52,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N52">
+        <f>IF(M52="",0,MAX(0,Settings!$B$5-M52)*F52/Settings!$B$4)</f>
+        <v>250376.58823529413</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>86</v>
       </c>
@@ -5384,8 +5815,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M53">
+        <f>_xlfn.XLOOKUP(I53,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N53">
+        <f>IF(M53="",0,MAX(0,Settings!$B$5-M53)*F53/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>250</v>
       </c>
@@ -5425,8 +5864,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M54">
+        <f>_xlfn.XLOOKUP(I54,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N54">
+        <f>IF(M54="",0,MAX(0,Settings!$B$5-M54)*F54/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>226</v>
       </c>
@@ -5466,8 +5913,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M55">
+        <f>_xlfn.XLOOKUP(I55,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N55">
+        <f>IF(M55="",0,MAX(0,Settings!$B$5-M55)*F55/Settings!$B$4)</f>
+        <v>244521.41176470587</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>272</v>
       </c>
@@ -5507,8 +5962,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M56">
+        <f>_xlfn.XLOOKUP(I56,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N56">
+        <f>IF(M56="",0,MAX(0,Settings!$B$5-M56)*F56/Settings!$B$4)</f>
+        <v>241970.23529411765</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>176</v>
       </c>
@@ -5548,8 +6011,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M57">
+        <f>_xlfn.XLOOKUP(I57,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N57">
+        <f>IF(M57="",0,MAX(0,Settings!$B$5-M57)*F57/Settings!$B$4)</f>
+        <v>120792</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>252</v>
       </c>
@@ -5589,8 +6060,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M58">
+        <f>_xlfn.XLOOKUP(I58,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N58">
+        <f>IF(M58="",0,MAX(0,Settings!$B$5-M58)*F58/Settings!$B$4)</f>
+        <v>116791.5294117647</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>90</v>
       </c>
@@ -5630,8 +6109,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M59">
+        <f>_xlfn.XLOOKUP(I59,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N59">
+        <f>IF(M59="",0,MAX(0,Settings!$B$5-M59)*F59/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>54</v>
       </c>
@@ -5671,8 +6158,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M60">
+        <f>_xlfn.XLOOKUP(I60,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N60">
+        <f>IF(M60="",0,MAX(0,Settings!$B$5-M60)*F60/Settings!$B$4)</f>
+        <v>225784.11764705883</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>164</v>
       </c>
@@ -5712,8 +6207,16 @@
         <f t="shared" si="3"/>
         <v>A</v>
       </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M61">
+        <f>_xlfn.XLOOKUP(I61,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N61">
+        <f>IF(M61="",0,MAX(0,Settings!$B$5-M61)*F61/Settings!$B$4)</f>
+        <v>225545.88235294117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>168</v>
       </c>
@@ -5753,8 +6256,16 @@
         <f t="shared" si="3"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M62">
+        <f>_xlfn.XLOOKUP(I62,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N62">
+        <f>IF(M62="",0,MAX(0,Settings!$B$5-M62)*F62/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>100</v>
       </c>
@@ -5794,8 +6305,16 @@
         <f t="shared" si="3"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M63">
+        <f>_xlfn.XLOOKUP(I63,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N63">
+        <f>IF(M63="",0,MAX(0,Settings!$B$5-M63)*F63/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -5835,8 +6354,16 @@
         <f t="shared" si="3"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M64">
+        <f>_xlfn.XLOOKUP(I64,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N64">
+        <f>IF(M64="",0,MAX(0,Settings!$B$5-M64)*F64/Settings!$B$4)</f>
+        <v>219250.23529411765</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>188</v>
       </c>
@@ -5876,8 +6403,16 @@
         <f t="shared" si="3"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M65">
+        <f>_xlfn.XLOOKUP(I65,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N65">
+        <f>IF(M65="",0,MAX(0,Settings!$B$5-M65)*F65/Settings!$B$4)</f>
+        <v>213996.4705882353</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>216</v>
       </c>
@@ -5917,8 +6452,16 @@
         <f t="shared" ref="L66:L97" si="5">IF(K66&lt;=80%,"A",IF(K66&lt;=95%,"B","C"))</f>
         <v>B</v>
       </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M66">
+        <f>_xlfn.XLOOKUP(I66,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N66">
+        <f>IF(M66="",0,MAX(0,Settings!$B$5-M66)*F66/Settings!$B$4)</f>
+        <v>209447.88235294117</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>246</v>
       </c>
@@ -5958,8 +6501,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M67">
+        <f>_xlfn.XLOOKUP(I67,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N67">
+        <f>IF(M67="",0,MAX(0,Settings!$B$5-M67)*F67/Settings!$B$4)</f>
+        <v>203225.88235294117</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>152</v>
       </c>
@@ -5999,8 +6550,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M68">
+        <f>_xlfn.XLOOKUP(I68,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N68">
+        <f>IF(M68="",0,MAX(0,Settings!$B$5-M68)*F68/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>210</v>
       </c>
@@ -6040,8 +6599,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M69">
+        <f>_xlfn.XLOOKUP(I69,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N69">
+        <f>IF(M69="",0,MAX(0,Settings!$B$5-M69)*F69/Settings!$B$4)</f>
+        <v>199281.17647058822</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>208</v>
       </c>
@@ -6081,8 +6648,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M70">
+        <f>_xlfn.XLOOKUP(I70,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N70">
+        <f>IF(M70="",0,MAX(0,Settings!$B$5-M70)*F70/Settings!$B$4)</f>
+        <v>95628.647058823524</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>212</v>
       </c>
@@ -6122,8 +6697,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M71">
+        <f>_xlfn.XLOOKUP(I71,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N71">
+        <f>IF(M71="",0,MAX(0,Settings!$B$5-M71)*F71/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -6163,8 +6746,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M72">
+        <f>_xlfn.XLOOKUP(I72,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N72">
+        <f>IF(M72="",0,MAX(0,Settings!$B$5-M72)*F72/Settings!$B$4)</f>
+        <v>181706.4705882353</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>104</v>
       </c>
@@ -6204,8 +6795,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M73">
+        <f>_xlfn.XLOOKUP(I73,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N73">
+        <f>IF(M73="",0,MAX(0,Settings!$B$5-M73)*F73/Settings!$B$4)</f>
+        <v>180252.35294117648</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>200</v>
       </c>
@@ -6245,8 +6844,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M74">
+        <f>_xlfn.XLOOKUP(I74,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N74">
+        <f>IF(M74="",0,MAX(0,Settings!$B$5-M74)*F74/Settings!$B$4)</f>
+        <v>174032</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>49</v>
       </c>
@@ -6286,8 +6893,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M75">
+        <f>_xlfn.XLOOKUP(I75,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N75">
+        <f>IF(M75="",0,MAX(0,Settings!$B$5-M75)*F75/Settings!$B$4)</f>
+        <v>165478.11764705883</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>144</v>
       </c>
@@ -6327,8 +6942,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M76">
+        <f>_xlfn.XLOOKUP(I76,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N76">
+        <f>IF(M76="",0,MAX(0,Settings!$B$5-M76)*F76/Settings!$B$4)</f>
+        <v>165354</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>118</v>
       </c>
@@ -6368,8 +6991,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M77">
+        <f>_xlfn.XLOOKUP(I77,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N77">
+        <f>IF(M77="",0,MAX(0,Settings!$B$5-M77)*F77/Settings!$B$4)</f>
+        <v>152103.76470588235</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -6409,8 +7040,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M78" t="str">
+        <f>_xlfn.XLOOKUP(I78,Terms!A:A,Terms!C:C,"")</f>
+        <v/>
+      </c>
+      <c r="N78">
+        <f>IF(M78="",0,MAX(0,Settings!$B$5-M78)*F78/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>194</v>
       </c>
@@ -6450,8 +7089,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M79">
+        <f>_xlfn.XLOOKUP(I79,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N79">
+        <f>IF(M79="",0,MAX(0,Settings!$B$5-M79)*F79/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>178</v>
       </c>
@@ -6491,8 +7138,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M80">
+        <f>_xlfn.XLOOKUP(I80,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N80">
+        <f>IF(M80="",0,MAX(0,Settings!$B$5-M80)*F80/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>116</v>
       </c>
@@ -6532,8 +7187,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M81">
+        <f>_xlfn.XLOOKUP(I81,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N81">
+        <f>IF(M81="",0,MAX(0,Settings!$B$5-M81)*F81/Settings!$B$4)</f>
+        <v>133968.11764705883</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>264</v>
       </c>
@@ -6573,8 +7236,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M82">
+        <f>_xlfn.XLOOKUP(I82,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N82">
+        <f>IF(M82="",0,MAX(0,Settings!$B$5-M82)*F82/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>162</v>
       </c>
@@ -6614,8 +7285,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M83">
+        <f>_xlfn.XLOOKUP(I83,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N83">
+        <f>IF(M83="",0,MAX(0,Settings!$B$5-M83)*F83/Settings!$B$4)</f>
+        <v>65396.76470588235</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>218</v>
       </c>
@@ -6655,8 +7334,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M84">
+        <f>_xlfn.XLOOKUP(I84,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N84">
+        <f>IF(M84="",0,MAX(0,Settings!$B$5-M84)*F84/Settings!$B$4)</f>
+        <v>64341.411764705881</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>56</v>
       </c>
@@ -6696,8 +7383,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M85">
+        <f>_xlfn.XLOOKUP(I85,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N85">
+        <f>IF(M85="",0,MAX(0,Settings!$B$5-M85)*F85/Settings!$B$4)</f>
+        <v>124886.58823529411</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>130</v>
       </c>
@@ -6737,8 +7432,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M86">
+        <f>_xlfn.XLOOKUP(I86,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N86">
+        <f>IF(M86="",0,MAX(0,Settings!$B$5-M86)*F86/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>184</v>
       </c>
@@ -6778,8 +7481,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M87">
+        <f>_xlfn.XLOOKUP(I87,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N87">
+        <f>IF(M87="",0,MAX(0,Settings!$B$5-M87)*F87/Settings!$B$4)</f>
+        <v>61030.058823529413</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -6819,8 +7530,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M88">
+        <f>_xlfn.XLOOKUP(I88,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N88">
+        <f>IF(M88="",0,MAX(0,Settings!$B$5-M88)*F88/Settings!$B$4)</f>
+        <v>119036.4705882353</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>166</v>
       </c>
@@ -6860,8 +7579,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M89">
+        <f>_xlfn.XLOOKUP(I89,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N89">
+        <f>IF(M89="",0,MAX(0,Settings!$B$5-M89)*F89/Settings!$B$4)</f>
+        <v>118352.58823529411</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>170</v>
       </c>
@@ -6901,8 +7628,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M90">
+        <f>_xlfn.XLOOKUP(I90,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N90">
+        <f>IF(M90="",0,MAX(0,Settings!$B$5-M90)*F90/Settings!$B$4)</f>
+        <v>58680</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>64</v>
       </c>
@@ -6942,8 +7677,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M91">
+        <f>_xlfn.XLOOKUP(I91,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N91">
+        <f>IF(M91="",0,MAX(0,Settings!$B$5-M91)*F91/Settings!$B$4)</f>
+        <v>114362.94117647059</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>98</v>
       </c>
@@ -6983,8 +7726,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M92">
+        <f>_xlfn.XLOOKUP(I92,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N92">
+        <f>IF(M92="",0,MAX(0,Settings!$B$5-M92)*F92/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>156</v>
       </c>
@@ -7024,8 +7775,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M93" t="str">
+        <f>_xlfn.XLOOKUP(I93,Terms!A:A,Terms!C:C,"")</f>
+        <v/>
+      </c>
+      <c r="N93">
+        <f>IF(M93="",0,MAX(0,Settings!$B$5-M93)*F93/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>40</v>
       </c>
@@ -7065,8 +7824,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M94">
+        <f>_xlfn.XLOOKUP(I94,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N94">
+        <f>IF(M94="",0,MAX(0,Settings!$B$5-M94)*F94/Settings!$B$4)</f>
+        <v>102606.82352941176</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>126</v>
       </c>
@@ -7106,8 +7873,16 @@
         <f t="shared" si="5"/>
         <v>B</v>
       </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M95">
+        <f>_xlfn.XLOOKUP(I95,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N95">
+        <f>IF(M95="",0,MAX(0,Settings!$B$5-M95)*F95/Settings!$B$4)</f>
+        <v>99885.882352941175</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>146</v>
       </c>
@@ -7147,8 +7922,16 @@
         <f t="shared" si="5"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M96">
+        <f>_xlfn.XLOOKUP(I96,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N96">
+        <f>IF(M96="",0,MAX(0,Settings!$B$5-M96)*F96/Settings!$B$4)</f>
+        <v>99731.058823529413</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>254</v>
       </c>
@@ -7188,8 +7971,16 @@
         <f t="shared" si="5"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M97">
+        <f>_xlfn.XLOOKUP(I97,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N97">
+        <f>IF(M97="",0,MAX(0,Settings!$B$5-M97)*F97/Settings!$B$4)</f>
+        <v>99695.294117647063</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>230</v>
       </c>
@@ -7229,8 +8020,16 @@
         <f t="shared" ref="L98:L121" si="7">IF(K98&lt;=80%,"A",IF(K98&lt;=95%,"B","C"))</f>
         <v>C</v>
       </c>
-    </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M98">
+        <f>_xlfn.XLOOKUP(I98,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N98">
+        <f>IF(M98="",0,MAX(0,Settings!$B$5-M98)*F98/Settings!$B$4)</f>
+        <v>49466.705882352944</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>262</v>
       </c>
@@ -7270,8 +8069,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M99">
+        <f>_xlfn.XLOOKUP(I99,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N99">
+        <f>IF(M99="",0,MAX(0,Settings!$B$5-M99)*F99/Settings!$B$4)</f>
+        <v>97918.705882352937</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>138</v>
       </c>
@@ -7311,8 +8118,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M100">
+        <f>_xlfn.XLOOKUP(I100,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N100">
+        <f>IF(M100="",0,MAX(0,Settings!$B$5-M100)*F100/Settings!$B$4)</f>
+        <v>45881.294117647056</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>174</v>
       </c>
@@ -7352,8 +8167,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M101">
+        <f>_xlfn.XLOOKUP(I101,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N101">
+        <f>IF(M101="",0,MAX(0,Settings!$B$5-M101)*F101/Settings!$B$4)</f>
+        <v>83150.941176470587</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>122</v>
       </c>
@@ -7393,8 +8216,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M102">
+        <f>_xlfn.XLOOKUP(I102,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N102">
+        <f>IF(M102="",0,MAX(0,Settings!$B$5-M102)*F102/Settings!$B$4)</f>
+        <v>40700.76470588235</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>232</v>
       </c>
@@ -7434,8 +8265,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M103">
+        <f>_xlfn.XLOOKUP(I103,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N103">
+        <f>IF(M103="",0,MAX(0,Settings!$B$5-M103)*F103/Settings!$B$4)</f>
+        <v>38816.823529411762</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>124</v>
       </c>
@@ -7475,8 +8314,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M104">
+        <f>_xlfn.XLOOKUP(I104,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N104">
+        <f>IF(M104="",0,MAX(0,Settings!$B$5-M104)*F104/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>244</v>
       </c>
@@ -7516,8 +8363,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M105">
+        <f>_xlfn.XLOOKUP(I105,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N105">
+        <f>IF(M105="",0,MAX(0,Settings!$B$5-M105)*F105/Settings!$B$4)</f>
+        <v>76645.647058823524</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>82</v>
       </c>
@@ -7557,8 +8412,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M106">
+        <f>_xlfn.XLOOKUP(I106,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N106">
+        <f>IF(M106="",0,MAX(0,Settings!$B$5-M106)*F106/Settings!$B$4)</f>
+        <v>76434.117647058825</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>270</v>
       </c>
@@ -7598,8 +8461,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M107">
+        <f>_xlfn.XLOOKUP(I107,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N107">
+        <f>IF(M107="",0,MAX(0,Settings!$B$5-M107)*F107/Settings!$B$4)</f>
+        <v>74183.529411764699</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>222</v>
       </c>
@@ -7639,8 +8510,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M108">
+        <f>_xlfn.XLOOKUP(I108,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N108">
+        <f>IF(M108="",0,MAX(0,Settings!$B$5-M108)*F108/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>66</v>
       </c>
@@ -7680,8 +8559,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M109">
+        <f>_xlfn.XLOOKUP(I109,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N109">
+        <f>IF(M109="",0,MAX(0,Settings!$B$5-M109)*F109/Settings!$B$4)</f>
+        <v>31949.176470588234</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>160</v>
       </c>
@@ -7721,8 +8608,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M110">
+        <f>_xlfn.XLOOKUP(I110,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N110">
+        <f>IF(M110="",0,MAX(0,Settings!$B$5-M110)*F110/Settings!$B$4)</f>
+        <v>62975.647058823532</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>240</v>
       </c>
@@ -7762,8 +8657,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M111">
+        <f>_xlfn.XLOOKUP(I111,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N111">
+        <f>IF(M111="",0,MAX(0,Settings!$B$5-M111)*F111/Settings!$B$4)</f>
+        <v>59749.058823529413</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>242</v>
       </c>
@@ -7803,8 +8706,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M112">
+        <f>_xlfn.XLOOKUP(I112,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N112">
+        <f>IF(M112="",0,MAX(0,Settings!$B$5-M112)*F112/Settings!$B$4)</f>
+        <v>25067.294117647059</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>31</v>
       </c>
@@ -7844,8 +8755,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M113">
+        <f>_xlfn.XLOOKUP(I113,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N113">
+        <f>IF(M113="",0,MAX(0,Settings!$B$5-M113)*F113/Settings!$B$4)</f>
+        <v>49458.705882352944</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>112</v>
       </c>
@@ -7885,8 +8804,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M114">
+        <f>_xlfn.XLOOKUP(I114,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N114">
+        <f>IF(M114="",0,MAX(0,Settings!$B$5-M114)*F114/Settings!$B$4)</f>
+        <v>24429.176470588234</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>224</v>
       </c>
@@ -7926,8 +8853,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M115">
+        <f>_xlfn.XLOOKUP(I115,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N115">
+        <f>IF(M115="",0,MAX(0,Settings!$B$5-M115)*F115/Settings!$B$4)</f>
+        <v>48082.705882352944</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>142</v>
       </c>
@@ -7967,8 +8902,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M116">
+        <f>_xlfn.XLOOKUP(I116,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N116">
+        <f>IF(M116="",0,MAX(0,Settings!$B$5-M116)*F116/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>37</v>
       </c>
@@ -8008,8 +8951,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M117">
+        <f>_xlfn.XLOOKUP(I117,Terms!A:A,Terms!C:C,"")</f>
+        <v>60</v>
+      </c>
+      <c r="N117">
+        <f>IF(M117="",0,MAX(0,Settings!$B$5-M117)*F117/Settings!$B$4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>248</v>
       </c>
@@ -8049,8 +9000,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M118">
+        <f>_xlfn.XLOOKUP(I118,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N118">
+        <f>IF(M118="",0,MAX(0,Settings!$B$5-M118)*F118/Settings!$B$4)</f>
+        <v>45600.588235294119</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>256</v>
       </c>
@@ -8090,8 +9049,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M119">
+        <f>_xlfn.XLOOKUP(I119,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N119">
+        <f>IF(M119="",0,MAX(0,Settings!$B$5-M119)*F119/Settings!$B$4)</f>
+        <v>37932.470588235294</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>140</v>
       </c>
@@ -8131,8 +9098,16 @@
         <f t="shared" si="7"/>
         <v>C</v>
       </c>
-    </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M120">
+        <f>_xlfn.XLOOKUP(I120,Terms!A:A,Terms!C:C,"")</f>
+        <v>45</v>
+      </c>
+      <c r="N120">
+        <f>IF(M120="",0,MAX(0,Settings!$B$5-M120)*F120/Settings!$B$4)</f>
+        <v>16990.117647058825</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>182</v>
       </c>
@@ -8171,6 +9146,14 @@
       <c r="L121" t="str">
         <f t="shared" si="7"/>
         <v>C</v>
+      </c>
+      <c r="M121">
+        <f>_xlfn.XLOOKUP(I121,Terms!A:A,Terms!C:C,"")</f>
+        <v>30</v>
+      </c>
+      <c r="N121">
+        <f>IF(M121="",0,MAX(0,Settings!$B$5-M121)*F121/Settings!$B$4)</f>
+        <v>31964.588235294119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M6 step 3c (part 2): cash discount potential and summary KPIs (cash effect, discount, suppliers and spend without payment terms)
</commit_message>
<xml_diff>
--- a/excel/Spend_Analysis.xlsx
+++ b/excel/Spend_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC0AB29-2118-CC40-8BC5-DBFA9AD6005B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94629A47-E9D3-F848-AECA-3DE49BB99AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suppliers" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="313">
   <si>
     <t>Golden ID</t>
   </si>
@@ -963,17 +963,33 @@
   </si>
   <si>
     <t>Cash effect (EUR)</t>
+  </si>
+  <si>
+    <t>Discount (EUR)</t>
+  </si>
+  <si>
+    <t>Cash effect, 60-day terms (EUR)</t>
+  </si>
+  <si>
+    <t>Cash discount potential (EUR)</t>
+  </si>
+  <si>
+    <t>Suppliers without payment terms</t>
+  </si>
+  <si>
+    <t>Spend without payment terms (EUR)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1001,6 +1017,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1024,11 +1046,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1044,12 +1067,19 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -2894,12 +2924,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSpend" displayName="tblSpend" ref="A1:N121">
-  <autoFilter ref="A1:N121" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblSpend" displayName="tblSpend" ref="A1:O121">
+  <autoFilter ref="A1:O121" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I121">
     <sortCondition descending="1" ref="F1:F121"/>
   </sortState>
-  <tableColumns count="14">
+  <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Golden ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Supplier"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Country"/>
@@ -2912,17 +2942,20 @@
     <tableColumn id="10" xr3:uid="{5D1E5103-053F-9149-A678-5C4D8626A5EA}" name="Spend share" dataCellStyle="Percent">
       <calculatedColumnFormula>F2/SUM($F$2:$F$121)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{B3C0593A-4800-A24E-858E-2C3789403277}" name="Cumulative share" dataDxfId="3">
+    <tableColumn id="11" xr3:uid="{B3C0593A-4800-A24E-858E-2C3789403277}" name="Cumulative share" dataDxfId="4">
       <calculatedColumnFormula>SUM($J$2:J2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{DFA46FC0-C59B-9B4C-8696-052595BBF44D}" name="ABC class" dataDxfId="2">
+    <tableColumn id="12" xr3:uid="{DFA46FC0-C59B-9B4C-8696-052595BBF44D}" name="ABC class" dataDxfId="3">
       <calculatedColumnFormula>IF(K2&lt;=80%,"A",IF(K2&lt;=95%,"B","C"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{A6793419-9AA1-3242-B71C-8AD377F8F478}" name="Net days" dataDxfId="1">
+    <tableColumn id="13" xr3:uid="{A6793419-9AA1-3242-B71C-8AD377F8F478}" name="Net days" dataDxfId="2">
       <calculatedColumnFormula>_xlfn.XLOOKUP(I2,Terms!A:A,Terms!C:C,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{0BFB64A9-2F55-0641-BBF7-61A0DC5F3A72}" name="Cash effect (EUR)" dataDxfId="0">
+    <tableColumn id="14" xr3:uid="{0BFB64A9-2F55-0641-BBF7-61A0DC5F3A72}" name="Cash effect (EUR)" dataDxfId="1">
       <calculatedColumnFormula>IF(M2="",0,MAX(0,Settings!$B$5-M2)*F2/Settings!$B$4)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="15" xr3:uid="{416A67A6-A46F-5A41-A253-2FCCBF2A67A5}" name="Discount (EUR)" dataDxfId="0">
+      <calculatedColumnFormula>F2*_xlfn.XLOOKUP(I2,Terms!A:A,Terms!D:D,0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3214,7 +3247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N121"/>
+  <dimension ref="A1:O121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
@@ -3230,9 +3263,10 @@
     <col min="12" max="12" width="13.6640625" customWidth="1"/>
     <col min="13" max="13" width="15.5" customWidth="1"/>
     <col min="14" max="14" width="21.1640625" customWidth="1"/>
+    <col min="15" max="15" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3275,8 +3309,11 @@
       <c r="N1" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O1" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>228</v>
       </c>
@@ -3324,8 +3361,12 @@
         <f>IF(M2="",0,MAX(0,Settings!$B$5-M2)*F2/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O2" s="11">
+        <f>F2*_xlfn.XLOOKUP(I2,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>61</v>
       </c>
@@ -3373,8 +3414,12 @@
         <f>IF(M3="",0,MAX(0,Settings!$B$5-M3)*F3/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O3" s="11">
+        <f>F3*_xlfn.XLOOKUP(I3,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>236</v>
       </c>
@@ -3422,8 +3467,12 @@
         <f>IF(M4="",0,MAX(0,Settings!$B$5-M4)*F4/Settings!$B$4)</f>
         <v>928559.4117647059</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O4" s="11">
+        <f>F4*_xlfn.XLOOKUP(I4,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>136</v>
       </c>
@@ -3471,8 +3520,12 @@
         <f>IF(M5="",0,MAX(0,Settings!$B$5-M5)*F5/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O5" s="11">
+        <f>F5*_xlfn.XLOOKUP(I5,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -3520,8 +3573,12 @@
         <f>IF(M6="",0,MAX(0,Settings!$B$5-M6)*F6/Settings!$B$4)</f>
         <v>412735.5882352941</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O6" s="11">
+        <f>F6*_xlfn.XLOOKUP(I6,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>198</v>
       </c>
@@ -3569,8 +3626,12 @@
         <f>IF(M7="",0,MAX(0,Settings!$B$5-M7)*F7/Settings!$B$4)</f>
         <v>775416.4705882353</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O7" s="11">
+        <f>F7*_xlfn.XLOOKUP(I7,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>238</v>
       </c>
@@ -3618,8 +3679,12 @@
         <f>IF(M8="",0,MAX(0,Settings!$B$5-M8)*F8/Settings!$B$4)</f>
         <v>765748.23529411759</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O8" s="11">
+        <f>F8*_xlfn.XLOOKUP(I8,Terms!A:A,Terms!D:D,0)</f>
+        <v>130177.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>120</v>
       </c>
@@ -3667,8 +3732,12 @@
         <f>IF(M9="",0,MAX(0,Settings!$B$5-M9)*F9/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O9" s="11">
+        <f>F9*_xlfn.XLOOKUP(I9,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>158</v>
       </c>
@@ -3716,8 +3785,12 @@
         <f>IF(M10="",0,MAX(0,Settings!$B$5-M10)*F10/Settings!$B$4)</f>
         <v>377947.0588235294</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O10" s="11">
+        <f>F10*_xlfn.XLOOKUP(I10,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>220</v>
       </c>
@@ -3765,8 +3838,12 @@
         <f>IF(M11="",0,MAX(0,Settings!$B$5-M11)*F11/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O11" s="11">
+        <f>F11*_xlfn.XLOOKUP(I11,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -3814,8 +3891,12 @@
         <f>IF(M12="",0,MAX(0,Settings!$B$5-M12)*F12/Settings!$B$4)</f>
         <v>351134.23529411765</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O12" s="11">
+        <f>F12*_xlfn.XLOOKUP(I12,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>266</v>
       </c>
@@ -3863,8 +3944,12 @@
         <f>IF(M13="",0,MAX(0,Settings!$B$5-M13)*F13/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O13" s="11">
+        <f>F13*_xlfn.XLOOKUP(I13,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>206</v>
       </c>
@@ -3912,8 +3997,12 @@
         <f>IF(M14="",0,MAX(0,Settings!$B$5-M14)*F14/Settings!$B$4)</f>
         <v>682780.3529411765</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O14" s="11">
+        <f>F14*_xlfn.XLOOKUP(I14,Terms!A:A,Terms!D:D,0)</f>
+        <v>116072.66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>180</v>
       </c>
@@ -3961,8 +4050,12 @@
         <f>IF(M15="",0,MAX(0,Settings!$B$5-M15)*F15/Settings!$B$4)</f>
         <v>650454</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O15" s="11">
+        <f>F15*_xlfn.XLOOKUP(I15,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>260</v>
       </c>
@@ -4010,8 +4103,12 @@
         <f>IF(M16="",0,MAX(0,Settings!$B$5-M16)*F16/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O16" s="11">
+        <f>F16*_xlfn.XLOOKUP(I16,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>172</v>
       </c>
@@ -4059,8 +4156,12 @@
         <f>IF(M17="",0,MAX(0,Settings!$B$5-M17)*F17/Settings!$B$4)</f>
         <v>574860.9411764706</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O17" s="11">
+        <f>F17*_xlfn.XLOOKUP(I17,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>76</v>
       </c>
@@ -4108,8 +4209,12 @@
         <f>IF(M18="",0,MAX(0,Settings!$B$5-M18)*F18/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O18" s="11">
+        <f>F18*_xlfn.XLOOKUP(I18,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -4157,8 +4262,12 @@
         <f>IF(M19="",0,MAX(0,Settings!$B$5-M19)*F19/Settings!$B$4)</f>
         <v>266302.64705882355</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O19" s="11">
+        <f>F19*_xlfn.XLOOKUP(I19,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>128</v>
       </c>
@@ -4206,8 +4315,12 @@
         <f>IF(M20="",0,MAX(0,Settings!$B$5-M20)*F20/Settings!$B$4)</f>
         <v>265671.70588235295</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O20" s="11">
+        <f>F20*_xlfn.XLOOKUP(I20,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>148</v>
       </c>
@@ -4255,8 +4368,12 @@
         <f>IF(M21="",0,MAX(0,Settings!$B$5-M21)*F21/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O21" s="11">
+        <f>F21*_xlfn.XLOOKUP(I21,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>192</v>
       </c>
@@ -4304,8 +4421,12 @@
         <f>IF(M22="",0,MAX(0,Settings!$B$5-M22)*F22/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O22" s="11">
+        <f>F22*_xlfn.XLOOKUP(I22,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>196</v>
       </c>
@@ -4353,8 +4474,12 @@
         <f>IF(M23="",0,MAX(0,Settings!$B$5-M23)*F23/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O23" s="11">
+        <f>F23*_xlfn.XLOOKUP(I23,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>15</v>
       </c>
@@ -4402,8 +4527,12 @@
         <f>IF(M24="",0,MAX(0,Settings!$B$5-M24)*F24/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O24" s="11">
+        <f>F24*_xlfn.XLOOKUP(I24,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>234</v>
       </c>
@@ -4451,8 +4580,12 @@
         <f>IF(M25="",0,MAX(0,Settings!$B$5-M25)*F25/Settings!$B$4)</f>
         <v>445921.0588235294</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O25" s="11">
+        <f>F25*_xlfn.XLOOKUP(I25,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>268</v>
       </c>
@@ -4500,8 +4633,12 @@
         <f>IF(M26="",0,MAX(0,Settings!$B$5-M26)*F26/Settings!$B$4)</f>
         <v>431708.5882352941</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O26" s="11">
+        <f>F26*_xlfn.XLOOKUP(I26,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>190</v>
       </c>
@@ -4549,8 +4686,12 @@
         <f>IF(M27="",0,MAX(0,Settings!$B$5-M27)*F27/Settings!$B$4)</f>
         <v>418819.17647058825</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O27" s="11">
+        <f>F27*_xlfn.XLOOKUP(I27,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>80</v>
       </c>
@@ -4598,8 +4739,12 @@
         <f>IF(M28="",0,MAX(0,Settings!$B$5-M28)*F28/Settings!$B$4)</f>
         <v>410567.0588235294</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O28" s="11">
+        <f>F28*_xlfn.XLOOKUP(I28,Terms!A:A,Terms!D:D,0)</f>
+        <v>69796.399999999994</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>96</v>
       </c>
@@ -4647,8 +4792,12 @@
         <f>IF(M29="",0,MAX(0,Settings!$B$5-M29)*F29/Settings!$B$4)</f>
         <v>203575.88235294117</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O29" s="11">
+        <f>F29*_xlfn.XLOOKUP(I29,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>202</v>
       </c>
@@ -4696,8 +4845,12 @@
         <f>IF(M30="",0,MAX(0,Settings!$B$5-M30)*F30/Settings!$B$4)</f>
         <v>403524</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O30" s="11">
+        <f>F30*_xlfn.XLOOKUP(I30,Terms!A:A,Terms!D:D,0)</f>
+        <v>68599.08</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>108</v>
       </c>
@@ -4745,8 +4898,12 @@
         <f>IF(M31="",0,MAX(0,Settings!$B$5-M31)*F31/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O31" s="11">
+        <f>F31*_xlfn.XLOOKUP(I31,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>106</v>
       </c>
@@ -4794,8 +4951,12 @@
         <f>IF(M32="",0,MAX(0,Settings!$B$5-M32)*F32/Settings!$B$4)</f>
         <v>365260</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O32" s="11">
+        <f>F32*_xlfn.XLOOKUP(I32,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>204</v>
       </c>
@@ -4843,8 +5004,12 @@
         <f>IF(M33="",0,MAX(0,Settings!$B$5-M33)*F33/Settings!$B$4)</f>
         <v>363602.5882352941</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O33" s="11">
+        <f>F33*_xlfn.XLOOKUP(I33,Terms!A:A,Terms!D:D,0)</f>
+        <v>61812.44</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>88</v>
       </c>
@@ -4892,8 +5057,12 @@
         <f>IF(M34="",0,MAX(0,Settings!$B$5-M34)*F34/Settings!$B$4)</f>
         <v>356528.5882352941</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O34" s="11">
+        <f>F34*_xlfn.XLOOKUP(I34,Terms!A:A,Terms!D:D,0)</f>
+        <v>60609.86</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>59</v>
       </c>
@@ -4941,8 +5110,12 @@
         <f>IF(M35="",0,MAX(0,Settings!$B$5-M35)*F35/Settings!$B$4)</f>
         <v>348141.29411764705</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O35" s="11">
+        <f>F35*_xlfn.XLOOKUP(I35,Terms!A:A,Terms!D:D,0)</f>
+        <v>59184.020000000004</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -4990,8 +5163,12 @@
         <f>IF(M36="",0,MAX(0,Settings!$B$5-M36)*F36/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O36" s="11">
+        <f>F36*_xlfn.XLOOKUP(I36,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>214</v>
       </c>
@@ -5039,8 +5216,12 @@
         <f>IF(M37="",0,MAX(0,Settings!$B$5-M37)*F37/Settings!$B$4)</f>
         <v>343931.4117647059</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O37" s="11">
+        <f>F37*_xlfn.XLOOKUP(I37,Terms!A:A,Terms!D:D,0)</f>
+        <v>58468.340000000004</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>26</v>
       </c>
@@ -5088,8 +5269,12 @@
         <f>IF(M38="",0,MAX(0,Settings!$B$5-M38)*F38/Settings!$B$4)</f>
         <v>339123.76470588235</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O38" s="11">
+        <f>F38*_xlfn.XLOOKUP(I38,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -5137,8 +5322,12 @@
         <f>IF(M39="",0,MAX(0,Settings!$B$5-M39)*F39/Settings!$B$4)</f>
         <v>337843.76470588235</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O39" s="11">
+        <f>F39*_xlfn.XLOOKUP(I39,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>150</v>
       </c>
@@ -5186,8 +5375,12 @@
         <f>IF(M40="",0,MAX(0,Settings!$B$5-M40)*F40/Settings!$B$4)</f>
         <v>337105.8823529412</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O40" s="11">
+        <f>F40*_xlfn.XLOOKUP(I40,Terms!A:A,Terms!D:D,0)</f>
+        <v>57308</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -5235,8 +5428,12 @@
         <f>IF(M41="",0,MAX(0,Settings!$B$5-M41)*F41/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O41" s="11">
+        <f>F41*_xlfn.XLOOKUP(I41,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>132</v>
       </c>
@@ -5284,8 +5481,12 @@
         <f>IF(M42="",0,MAX(0,Settings!$B$5-M42)*F42/Settings!$B$4)</f>
         <v>317400.1176470588</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O42" s="11">
+        <f>F42*_xlfn.XLOOKUP(I42,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>154</v>
       </c>
@@ -5333,8 +5534,12 @@
         <f>IF(M43="",0,MAX(0,Settings!$B$5-M43)*F43/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O43" s="11">
+        <f>F43*_xlfn.XLOOKUP(I43,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>92</v>
       </c>
@@ -5382,8 +5587,12 @@
         <f>IF(M44="",0,MAX(0,Settings!$B$5-M44)*F44/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O44" s="11">
+        <f>F44*_xlfn.XLOOKUP(I44,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -5431,8 +5640,12 @@
         <f>IF(M45="",0,MAX(0,Settings!$B$5-M45)*F45/Settings!$B$4)</f>
         <v>145105.64705882352</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O45" s="11">
+        <f>F45*_xlfn.XLOOKUP(I45,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>102</v>
       </c>
@@ -5480,8 +5693,12 @@
         <f>IF(M46="",0,MAX(0,Settings!$B$5-M46)*F46/Settings!$B$4)</f>
         <v>286492.4705882353</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O46" s="11">
+        <f>F46*_xlfn.XLOOKUP(I46,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>258</v>
       </c>
@@ -5529,8 +5746,12 @@
         <f>IF(M47="",0,MAX(0,Settings!$B$5-M47)*F47/Settings!$B$4)</f>
         <v>136814.64705882352</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O47" s="11">
+        <f>F47*_xlfn.XLOOKUP(I47,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>110</v>
       </c>
@@ -5578,8 +5799,12 @@
         <f>IF(M48="",0,MAX(0,Settings!$B$5-M48)*F48/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O48" s="11">
+        <f>F48*_xlfn.XLOOKUP(I48,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>134</v>
       </c>
@@ -5627,8 +5852,12 @@
         <f>IF(M49="",0,MAX(0,Settings!$B$5-M49)*F49/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O49" s="11">
+        <f>F49*_xlfn.XLOOKUP(I49,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>94</v>
       </c>
@@ -5676,8 +5905,12 @@
         <f>IF(M50="",0,MAX(0,Settings!$B$5-M50)*F50/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O50" s="11">
+        <f>F50*_xlfn.XLOOKUP(I50,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>73</v>
       </c>
@@ -5725,8 +5958,12 @@
         <f>IF(M51="",0,MAX(0,Settings!$B$5-M51)*F51/Settings!$B$4)</f>
         <v>131488.76470588235</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O51" s="11">
+        <f>F51*_xlfn.XLOOKUP(I51,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>114</v>
       </c>
@@ -5774,8 +6011,12 @@
         <f>IF(M52="",0,MAX(0,Settings!$B$5-M52)*F52/Settings!$B$4)</f>
         <v>250376.58823529413</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O52" s="11">
+        <f>F52*_xlfn.XLOOKUP(I52,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>86</v>
       </c>
@@ -5823,8 +6064,12 @@
         <f>IF(M53="",0,MAX(0,Settings!$B$5-M53)*F53/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O53" s="11">
+        <f>F53*_xlfn.XLOOKUP(I53,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>250</v>
       </c>
@@ -5872,8 +6117,12 @@
         <f>IF(M54="",0,MAX(0,Settings!$B$5-M54)*F54/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O54" s="11">
+        <f>F54*_xlfn.XLOOKUP(I54,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>226</v>
       </c>
@@ -5921,8 +6170,12 @@
         <f>IF(M55="",0,MAX(0,Settings!$B$5-M55)*F55/Settings!$B$4)</f>
         <v>244521.41176470587</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O55" s="11">
+        <f>F55*_xlfn.XLOOKUP(I55,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>272</v>
       </c>
@@ -5970,8 +6223,12 @@
         <f>IF(M56="",0,MAX(0,Settings!$B$5-M56)*F56/Settings!$B$4)</f>
         <v>241970.23529411765</v>
       </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O56" s="11">
+        <f>F56*_xlfn.XLOOKUP(I56,Terms!A:A,Terms!D:D,0)</f>
+        <v>41134.94</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>176</v>
       </c>
@@ -6019,8 +6276,12 @@
         <f>IF(M57="",0,MAX(0,Settings!$B$5-M57)*F57/Settings!$B$4)</f>
         <v>120792</v>
       </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O57" s="11">
+        <f>F57*_xlfn.XLOOKUP(I57,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>252</v>
       </c>
@@ -6068,8 +6329,12 @@
         <f>IF(M58="",0,MAX(0,Settings!$B$5-M58)*F58/Settings!$B$4)</f>
         <v>116791.5294117647</v>
       </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O58" s="11">
+        <f>F58*_xlfn.XLOOKUP(I58,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>90</v>
       </c>
@@ -6117,8 +6382,12 @@
         <f>IF(M59="",0,MAX(0,Settings!$B$5-M59)*F59/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O59" s="11">
+        <f>F59*_xlfn.XLOOKUP(I59,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>54</v>
       </c>
@@ -6166,8 +6435,12 @@
         <f>IF(M60="",0,MAX(0,Settings!$B$5-M60)*F60/Settings!$B$4)</f>
         <v>225784.11764705883</v>
       </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O60" s="11">
+        <f>F60*_xlfn.XLOOKUP(I60,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>164</v>
       </c>
@@ -6215,8 +6488,12 @@
         <f>IF(M61="",0,MAX(0,Settings!$B$5-M61)*F61/Settings!$B$4)</f>
         <v>225545.88235294117</v>
       </c>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O61" s="11">
+        <f>F61*_xlfn.XLOOKUP(I61,Terms!A:A,Terms!D:D,0)</f>
+        <v>38342.800000000003</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>168</v>
       </c>
@@ -6264,8 +6541,12 @@
         <f>IF(M62="",0,MAX(0,Settings!$B$5-M62)*F62/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O62" s="11">
+        <f>F62*_xlfn.XLOOKUP(I62,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>100</v>
       </c>
@@ -6313,8 +6594,12 @@
         <f>IF(M63="",0,MAX(0,Settings!$B$5-M63)*F63/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O63" s="11">
+        <f>F63*_xlfn.XLOOKUP(I63,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -6362,8 +6647,12 @@
         <f>IF(M64="",0,MAX(0,Settings!$B$5-M64)*F64/Settings!$B$4)</f>
         <v>219250.23529411765</v>
       </c>
-    </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O64" s="11">
+        <f>F64*_xlfn.XLOOKUP(I64,Terms!A:A,Terms!D:D,0)</f>
+        <v>37272.54</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>188</v>
       </c>
@@ -6411,8 +6700,12 @@
         <f>IF(M65="",0,MAX(0,Settings!$B$5-M65)*F65/Settings!$B$4)</f>
         <v>213996.4705882353</v>
       </c>
-    </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O65" s="11">
+        <f>F65*_xlfn.XLOOKUP(I65,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>216</v>
       </c>
@@ -6460,8 +6753,12 @@
         <f>IF(M66="",0,MAX(0,Settings!$B$5-M66)*F66/Settings!$B$4)</f>
         <v>209447.88235294117</v>
       </c>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O66" s="11">
+        <f>F66*_xlfn.XLOOKUP(I66,Terms!A:A,Terms!D:D,0)</f>
+        <v>35606.14</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>246</v>
       </c>
@@ -6509,8 +6806,12 @@
         <f>IF(M67="",0,MAX(0,Settings!$B$5-M67)*F67/Settings!$B$4)</f>
         <v>203225.88235294117</v>
       </c>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O67" s="11">
+        <f>F67*_xlfn.XLOOKUP(I67,Terms!A:A,Terms!D:D,0)</f>
+        <v>34548.400000000001</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>152</v>
       </c>
@@ -6558,8 +6859,12 @@
         <f>IF(M68="",0,MAX(0,Settings!$B$5-M68)*F68/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O68" s="11">
+        <f>F68*_xlfn.XLOOKUP(I68,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>210</v>
       </c>
@@ -6607,8 +6912,12 @@
         <f>IF(M69="",0,MAX(0,Settings!$B$5-M69)*F69/Settings!$B$4)</f>
         <v>199281.17647058822</v>
       </c>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O69" s="11">
+        <f>F69*_xlfn.XLOOKUP(I69,Terms!A:A,Terms!D:D,0)</f>
+        <v>33877.800000000003</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>208</v>
       </c>
@@ -6656,8 +6965,12 @@
         <f>IF(M70="",0,MAX(0,Settings!$B$5-M70)*F70/Settings!$B$4)</f>
         <v>95628.647058823524</v>
       </c>
-    </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O70" s="11">
+        <f>F70*_xlfn.XLOOKUP(I70,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>212</v>
       </c>
@@ -6705,8 +7018,12 @@
         <f>IF(M71="",0,MAX(0,Settings!$B$5-M71)*F71/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O71" s="11">
+        <f>F71*_xlfn.XLOOKUP(I71,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -6754,8 +7071,12 @@
         <f>IF(M72="",0,MAX(0,Settings!$B$5-M72)*F72/Settings!$B$4)</f>
         <v>181706.4705882353</v>
       </c>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O72" s="11">
+        <f>F72*_xlfn.XLOOKUP(I72,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>104</v>
       </c>
@@ -6803,8 +7124,12 @@
         <f>IF(M73="",0,MAX(0,Settings!$B$5-M73)*F73/Settings!$B$4)</f>
         <v>180252.35294117648</v>
       </c>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O73" s="11">
+        <f>F73*_xlfn.XLOOKUP(I73,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>200</v>
       </c>
@@ -6852,8 +7177,12 @@
         <f>IF(M74="",0,MAX(0,Settings!$B$5-M74)*F74/Settings!$B$4)</f>
         <v>174032</v>
       </c>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O74" s="11">
+        <f>F74*_xlfn.XLOOKUP(I74,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>49</v>
       </c>
@@ -6901,8 +7230,12 @@
         <f>IF(M75="",0,MAX(0,Settings!$B$5-M75)*F75/Settings!$B$4)</f>
         <v>165478.11764705883</v>
       </c>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O75" s="11">
+        <f>F75*_xlfn.XLOOKUP(I75,Terms!A:A,Terms!D:D,0)</f>
+        <v>28131.279999999999</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>144</v>
       </c>
@@ -6950,8 +7283,12 @@
         <f>IF(M76="",0,MAX(0,Settings!$B$5-M76)*F76/Settings!$B$4)</f>
         <v>165354</v>
       </c>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O76" s="11">
+        <f>F76*_xlfn.XLOOKUP(I76,Terms!A:A,Terms!D:D,0)</f>
+        <v>28110.18</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>118</v>
       </c>
@@ -6999,8 +7336,12 @@
         <f>IF(M77="",0,MAX(0,Settings!$B$5-M77)*F77/Settings!$B$4)</f>
         <v>152103.76470588235</v>
       </c>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O77" s="11">
+        <f>F77*_xlfn.XLOOKUP(I77,Terms!A:A,Terms!D:D,0)</f>
+        <v>25857.64</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -7048,8 +7389,12 @@
         <f>IF(M78="",0,MAX(0,Settings!$B$5-M78)*F78/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O78" s="11">
+        <f>F78*_xlfn.XLOOKUP(I78,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>194</v>
       </c>
@@ -7097,8 +7442,12 @@
         <f>IF(M79="",0,MAX(0,Settings!$B$5-M79)*F79/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O79" s="11">
+        <f>F79*_xlfn.XLOOKUP(I79,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>178</v>
       </c>
@@ -7146,8 +7495,12 @@
         <f>IF(M80="",0,MAX(0,Settings!$B$5-M80)*F80/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O80" s="11">
+        <f>F80*_xlfn.XLOOKUP(I80,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>116</v>
       </c>
@@ -7195,8 +7548,12 @@
         <f>IF(M81="",0,MAX(0,Settings!$B$5-M81)*F81/Settings!$B$4)</f>
         <v>133968.11764705883</v>
       </c>
-    </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O81" s="11">
+        <f>F81*_xlfn.XLOOKUP(I81,Terms!A:A,Terms!D:D,0)</f>
+        <v>22774.58</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>264</v>
       </c>
@@ -7244,8 +7601,12 @@
         <f>IF(M82="",0,MAX(0,Settings!$B$5-M82)*F82/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O82" s="11">
+        <f>F82*_xlfn.XLOOKUP(I82,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>162</v>
       </c>
@@ -7293,8 +7654,12 @@
         <f>IF(M83="",0,MAX(0,Settings!$B$5-M83)*F83/Settings!$B$4)</f>
         <v>65396.76470588235</v>
       </c>
-    </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O83" s="11">
+        <f>F83*_xlfn.XLOOKUP(I83,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>218</v>
       </c>
@@ -7342,8 +7707,12 @@
         <f>IF(M84="",0,MAX(0,Settings!$B$5-M84)*F84/Settings!$B$4)</f>
         <v>64341.411764705881</v>
       </c>
-    </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O84" s="11">
+        <f>F84*_xlfn.XLOOKUP(I84,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>56</v>
       </c>
@@ -7391,8 +7760,12 @@
         <f>IF(M85="",0,MAX(0,Settings!$B$5-M85)*F85/Settings!$B$4)</f>
         <v>124886.58823529411</v>
       </c>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O85" s="11">
+        <f>F85*_xlfn.XLOOKUP(I85,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>130</v>
       </c>
@@ -7440,8 +7813,12 @@
         <f>IF(M86="",0,MAX(0,Settings!$B$5-M86)*F86/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O86" s="11">
+        <f>F86*_xlfn.XLOOKUP(I86,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>184</v>
       </c>
@@ -7489,8 +7866,12 @@
         <f>IF(M87="",0,MAX(0,Settings!$B$5-M87)*F87/Settings!$B$4)</f>
         <v>61030.058823529413</v>
       </c>
-    </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O87" s="11">
+        <f>F87*_xlfn.XLOOKUP(I87,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -7538,8 +7919,12 @@
         <f>IF(M88="",0,MAX(0,Settings!$B$5-M88)*F88/Settings!$B$4)</f>
         <v>119036.4705882353</v>
       </c>
-    </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O88" s="11">
+        <f>F88*_xlfn.XLOOKUP(I88,Terms!A:A,Terms!D:D,0)</f>
+        <v>20236.2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>166</v>
       </c>
@@ -7587,8 +7972,12 @@
         <f>IF(M89="",0,MAX(0,Settings!$B$5-M89)*F89/Settings!$B$4)</f>
         <v>118352.58823529411</v>
       </c>
-    </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O89" s="11">
+        <f>F89*_xlfn.XLOOKUP(I89,Terms!A:A,Terms!D:D,0)</f>
+        <v>20119.939999999999</v>
+      </c>
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>170</v>
       </c>
@@ -7636,8 +8025,12 @@
         <f>IF(M90="",0,MAX(0,Settings!$B$5-M90)*F90/Settings!$B$4)</f>
         <v>58680</v>
       </c>
-    </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O90" s="11">
+        <f>F90*_xlfn.XLOOKUP(I90,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>64</v>
       </c>
@@ -7685,8 +8078,12 @@
         <f>IF(M91="",0,MAX(0,Settings!$B$5-M91)*F91/Settings!$B$4)</f>
         <v>114362.94117647059</v>
       </c>
-    </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O91" s="11">
+        <f>F91*_xlfn.XLOOKUP(I91,Terms!A:A,Terms!D:D,0)</f>
+        <v>19441.7</v>
+      </c>
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>98</v>
       </c>
@@ -7734,8 +8131,12 @@
         <f>IF(M92="",0,MAX(0,Settings!$B$5-M92)*F92/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O92" s="11">
+        <f>F92*_xlfn.XLOOKUP(I92,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>156</v>
       </c>
@@ -7783,8 +8184,12 @@
         <f>IF(M93="",0,MAX(0,Settings!$B$5-M93)*F93/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O93" s="11">
+        <f>F93*_xlfn.XLOOKUP(I93,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>40</v>
       </c>
@@ -7832,8 +8237,12 @@
         <f>IF(M94="",0,MAX(0,Settings!$B$5-M94)*F94/Settings!$B$4)</f>
         <v>102606.82352941176</v>
       </c>
-    </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O94" s="11">
+        <f>F94*_xlfn.XLOOKUP(I94,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>126</v>
       </c>
@@ -7881,8 +8290,12 @@
         <f>IF(M95="",0,MAX(0,Settings!$B$5-M95)*F95/Settings!$B$4)</f>
         <v>99885.882352941175</v>
       </c>
-    </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O95" s="11">
+        <f>F95*_xlfn.XLOOKUP(I95,Terms!A:A,Terms!D:D,0)</f>
+        <v>16980.599999999999</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>146</v>
       </c>
@@ -7930,8 +8343,12 @@
         <f>IF(M96="",0,MAX(0,Settings!$B$5-M96)*F96/Settings!$B$4)</f>
         <v>99731.058823529413</v>
       </c>
-    </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O96" s="11">
+        <f>F96*_xlfn.XLOOKUP(I96,Terms!A:A,Terms!D:D,0)</f>
+        <v>16954.28</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>254</v>
       </c>
@@ -7979,8 +8396,12 @@
         <f>IF(M97="",0,MAX(0,Settings!$B$5-M97)*F97/Settings!$B$4)</f>
         <v>99695.294117647063</v>
       </c>
-    </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O97" s="11">
+        <f>F97*_xlfn.XLOOKUP(I97,Terms!A:A,Terms!D:D,0)</f>
+        <v>16948.2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>230</v>
       </c>
@@ -8028,8 +8449,12 @@
         <f>IF(M98="",0,MAX(0,Settings!$B$5-M98)*F98/Settings!$B$4)</f>
         <v>49466.705882352944</v>
       </c>
-    </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O98" s="11">
+        <f>F98*_xlfn.XLOOKUP(I98,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>262</v>
       </c>
@@ -8077,8 +8502,12 @@
         <f>IF(M99="",0,MAX(0,Settings!$B$5-M99)*F99/Settings!$B$4)</f>
         <v>97918.705882352937</v>
       </c>
-    </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O99" s="11">
+        <f>F99*_xlfn.XLOOKUP(I99,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>138</v>
       </c>
@@ -8126,8 +8555,12 @@
         <f>IF(M100="",0,MAX(0,Settings!$B$5-M100)*F100/Settings!$B$4)</f>
         <v>45881.294117647056</v>
       </c>
-    </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O100" s="11">
+        <f>F100*_xlfn.XLOOKUP(I100,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>174</v>
       </c>
@@ -8175,8 +8608,12 @@
         <f>IF(M101="",0,MAX(0,Settings!$B$5-M101)*F101/Settings!$B$4)</f>
         <v>83150.941176470587</v>
       </c>
-    </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O101" s="11">
+        <f>F101*_xlfn.XLOOKUP(I101,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>122</v>
       </c>
@@ -8224,8 +8661,12 @@
         <f>IF(M102="",0,MAX(0,Settings!$B$5-M102)*F102/Settings!$B$4)</f>
         <v>40700.76470588235</v>
       </c>
-    </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O102" s="11">
+        <f>F102*_xlfn.XLOOKUP(I102,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>232</v>
       </c>
@@ -8273,8 +8714,12 @@
         <f>IF(M103="",0,MAX(0,Settings!$B$5-M103)*F103/Settings!$B$4)</f>
         <v>38816.823529411762</v>
       </c>
-    </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O103" s="11">
+        <f>F103*_xlfn.XLOOKUP(I103,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>124</v>
       </c>
@@ -8322,8 +8767,12 @@
         <f>IF(M104="",0,MAX(0,Settings!$B$5-M104)*F104/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O104" s="11">
+        <f>F104*_xlfn.XLOOKUP(I104,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>244</v>
       </c>
@@ -8371,8 +8820,12 @@
         <f>IF(M105="",0,MAX(0,Settings!$B$5-M105)*F105/Settings!$B$4)</f>
         <v>76645.647058823524</v>
       </c>
-    </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O105" s="11">
+        <f>F105*_xlfn.XLOOKUP(I105,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>82</v>
       </c>
@@ -8420,8 +8873,12 @@
         <f>IF(M106="",0,MAX(0,Settings!$B$5-M106)*F106/Settings!$B$4)</f>
         <v>76434.117647058825</v>
       </c>
-    </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O106" s="11">
+        <f>F106*_xlfn.XLOOKUP(I106,Terms!A:A,Terms!D:D,0)</f>
+        <v>12993.800000000001</v>
+      </c>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>270</v>
       </c>
@@ -8469,8 +8926,12 @@
         <f>IF(M107="",0,MAX(0,Settings!$B$5-M107)*F107/Settings!$B$4)</f>
         <v>74183.529411764699</v>
       </c>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O107" s="11">
+        <f>F107*_xlfn.XLOOKUP(I107,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>222</v>
       </c>
@@ -8518,8 +8979,12 @@
         <f>IF(M108="",0,MAX(0,Settings!$B$5-M108)*F108/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O108" s="11">
+        <f>F108*_xlfn.XLOOKUP(I108,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>66</v>
       </c>
@@ -8567,8 +9032,12 @@
         <f>IF(M109="",0,MAX(0,Settings!$B$5-M109)*F109/Settings!$B$4)</f>
         <v>31949.176470588234</v>
       </c>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O109" s="11">
+        <f>F109*_xlfn.XLOOKUP(I109,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>160</v>
       </c>
@@ -8616,8 +9085,12 @@
         <f>IF(M110="",0,MAX(0,Settings!$B$5-M110)*F110/Settings!$B$4)</f>
         <v>62975.647058823532</v>
       </c>
-    </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O110" s="11">
+        <f>F110*_xlfn.XLOOKUP(I110,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>240</v>
       </c>
@@ -8665,8 +9138,12 @@
         <f>IF(M111="",0,MAX(0,Settings!$B$5-M111)*F111/Settings!$B$4)</f>
         <v>59749.058823529413</v>
       </c>
-    </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O111" s="11">
+        <f>F111*_xlfn.XLOOKUP(I111,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>242</v>
       </c>
@@ -8714,8 +9191,12 @@
         <f>IF(M112="",0,MAX(0,Settings!$B$5-M112)*F112/Settings!$B$4)</f>
         <v>25067.294117647059</v>
       </c>
-    </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O112" s="11">
+        <f>F112*_xlfn.XLOOKUP(I112,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>31</v>
       </c>
@@ -8763,8 +9244,12 @@
         <f>IF(M113="",0,MAX(0,Settings!$B$5-M113)*F113/Settings!$B$4)</f>
         <v>49458.705882352944</v>
       </c>
-    </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O113" s="11">
+        <f>F113*_xlfn.XLOOKUP(I113,Terms!A:A,Terms!D:D,0)</f>
+        <v>8407.98</v>
+      </c>
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>112</v>
       </c>
@@ -8812,8 +9297,12 @@
         <f>IF(M114="",0,MAX(0,Settings!$B$5-M114)*F114/Settings!$B$4)</f>
         <v>24429.176470588234</v>
       </c>
-    </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O114" s="11">
+        <f>F114*_xlfn.XLOOKUP(I114,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>224</v>
       </c>
@@ -8861,8 +9350,12 @@
         <f>IF(M115="",0,MAX(0,Settings!$B$5-M115)*F115/Settings!$B$4)</f>
         <v>48082.705882352944</v>
       </c>
-    </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O115" s="11">
+        <f>F115*_xlfn.XLOOKUP(I115,Terms!A:A,Terms!D:D,0)</f>
+        <v>8174.06</v>
+      </c>
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>142</v>
       </c>
@@ -8910,8 +9403,12 @@
         <f>IF(M116="",0,MAX(0,Settings!$B$5-M116)*F116/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O116" s="11">
+        <f>F116*_xlfn.XLOOKUP(I116,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>37</v>
       </c>
@@ -8959,8 +9456,12 @@
         <f>IF(M117="",0,MAX(0,Settings!$B$5-M117)*F117/Settings!$B$4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O117" s="11">
+        <f>F117*_xlfn.XLOOKUP(I117,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>248</v>
       </c>
@@ -9008,8 +9509,12 @@
         <f>IF(M118="",0,MAX(0,Settings!$B$5-M118)*F118/Settings!$B$4)</f>
         <v>45600.588235294119</v>
       </c>
-    </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O118" s="11">
+        <f>F118*_xlfn.XLOOKUP(I118,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>256</v>
       </c>
@@ -9057,8 +9562,12 @@
         <f>IF(M119="",0,MAX(0,Settings!$B$5-M119)*F119/Settings!$B$4)</f>
         <v>37932.470588235294</v>
       </c>
-    </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O119" s="11">
+        <f>F119*_xlfn.XLOOKUP(I119,Terms!A:A,Terms!D:D,0)</f>
+        <v>6448.52</v>
+      </c>
+    </row>
+    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>140</v>
       </c>
@@ -9106,8 +9615,12 @@
         <f>IF(M120="",0,MAX(0,Settings!$B$5-M120)*F120/Settings!$B$4)</f>
         <v>16990.117647058825</v>
       </c>
-    </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O120" s="11">
+        <f>F120*_xlfn.XLOOKUP(I120,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>182</v>
       </c>
@@ -9154,6 +9667,10 @@
       <c r="N121">
         <f>IF(M121="",0,MAX(0,Settings!$B$5-M121)*F121/Settings!$B$4)</f>
         <v>31964.588235294119</v>
+      </c>
+      <c r="O121" s="11">
+        <f>F121*_xlfn.XLOOKUP(I121,Terms!A:A,Terms!D:D,0)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9166,9 +9683,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD49C0F8-9F96-4F47-B62A-6FDD67704BE5}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="30.1640625" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
     <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
@@ -9283,6 +9802,42 @@
       </c>
       <c r="F7" s="10">
         <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>309</v>
+      </c>
+      <c r="B8" s="12">
+        <f>SUM(Suppliers!N:N)</f>
+        <v>18039476.176470581</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>310</v>
+      </c>
+      <c r="B9" s="12">
+        <f>SUM(Suppliers!O:O)</f>
+        <v>1154389.5800000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>311</v>
+      </c>
+      <c r="B10">
+        <f>COUNTIF(Suppliers!I:I,"missing")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B11" s="13">
+        <f>SUMIF(Suppliers!I:I,"missing",Suppliers!F:F)</f>
+        <v>12687450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>